<commit_message>
Fix scenario multiplier number format and update docstring row map
Co-authored-by: DejAmour <159169578+DejAmour@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/financial_model.xlsx
+++ b/financial_model.xlsx
@@ -26,12 +26,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="£#,##0.00"/>
     <numFmt numFmtId="166" formatCode="£#,##0"/>
-    <numFmt numFmtId="167" formatCode="0.0x"/>
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -150,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -187,9 +186,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1529,7 +1525,7 @@
           <t>Wind Turbine Capacity (MW, midpoint of 2–3 MW)</t>
         </is>
       </c>
-      <c r="C66" s="14" t="n">
+      <c r="C66" s="11" t="n">
         <v>2.5</v>
       </c>
     </row>
@@ -1571,14 +1567,14 @@
           <t>Reference:</t>
         </is>
       </c>
-      <c r="C70" s="15" t="inlineStr">
+      <c r="C70" s="14" t="inlineStr">
         <is>
           <t>UK DESNZ LCOE estimates — https://www.gov.uk/government/collections/energy-statistics</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="16" t="inlineStr">
+      <c r="A71" s="15" t="inlineStr">
         <is>
           <t>Note: kWh contracts assumed 10 years; model period = 5 years only. Ongoing revenues not modelled beyond 2030.</t>
         </is>
@@ -1622,7 +1618,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>SCENARIOS — TOTAL FUNDS RAISED</t>
         </is>
@@ -1636,7 +1632,7 @@
       <c r="H1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>Scenarios only affect Total Funds Raised. All other assumptions remain constant.</t>
         </is>
@@ -1657,7 +1653,7 @@
       <c r="H4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
@@ -1682,7 +1678,7 @@
       <c r="G5" s="9" t="n">
         <v>2030</v>
       </c>
-      <c r="H5" s="19" t="inlineStr">
+      <c r="H5" s="18" t="inlineStr">
         <is>
           <t>Multiplier</t>
         </is>
@@ -1699,27 +1695,27 @@
           <t>Base × 0.6  (40% reduction in Funds Raised)</t>
         </is>
       </c>
-      <c r="C6" s="20">
+      <c r="C6" s="19">
         <f>Assumptions!C16*Assumptions!C19</f>
         <v/>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="19">
         <f>Assumptions!D16*Assumptions!C19</f>
         <v/>
       </c>
-      <c r="E6" s="20">
+      <c r="E6" s="19">
         <f>Assumptions!E16*Assumptions!C19</f>
         <v/>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="19">
         <f>Assumptions!F16*Assumptions!C19</f>
         <v/>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="19">
         <f>Assumptions!G16*Assumptions!C19</f>
         <v/>
       </c>
-      <c r="H6" s="21" t="inlineStr">
+      <c r="H6" s="20" t="inlineStr">
         <is>
           <t>0.6</t>
         </is>
@@ -1736,27 +1732,27 @@
           <t>Central assumption — as per business plan</t>
         </is>
       </c>
-      <c r="C7" s="20">
+      <c r="C7" s="19">
         <f>Assumptions!C16</f>
         <v/>
       </c>
-      <c r="D7" s="20">
+      <c r="D7" s="19">
         <f>Assumptions!D16</f>
         <v/>
       </c>
-      <c r="E7" s="20">
+      <c r="E7" s="19">
         <f>Assumptions!E16</f>
         <v/>
       </c>
-      <c r="F7" s="20">
+      <c r="F7" s="19">
         <f>Assumptions!F16</f>
         <v/>
       </c>
-      <c r="G7" s="20">
+      <c r="G7" s="19">
         <f>Assumptions!G16</f>
         <v/>
       </c>
-      <c r="H7" s="21" t="inlineStr">
+      <c r="H7" s="20" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
@@ -1773,27 +1769,27 @@
           <t>Base × 1.4  (40% uplift in Funds Raised)</t>
         </is>
       </c>
-      <c r="C8" s="20">
+      <c r="C8" s="19">
         <f>Assumptions!C16*Assumptions!C20</f>
         <v/>
       </c>
-      <c r="D8" s="20">
+      <c r="D8" s="19">
         <f>Assumptions!D16*Assumptions!C20</f>
         <v/>
       </c>
-      <c r="E8" s="20">
+      <c r="E8" s="19">
         <f>Assumptions!E16*Assumptions!C20</f>
         <v/>
       </c>
-      <c r="F8" s="20">
+      <c r="F8" s="19">
         <f>Assumptions!F16*Assumptions!C20</f>
         <v/>
       </c>
-      <c r="G8" s="20">
+      <c r="G8" s="19">
         <f>Assumptions!G16*Assumptions!C20</f>
         <v/>
       </c>
-      <c r="H8" s="21" t="inlineStr">
+      <c r="H8" s="20" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
@@ -1819,7 +1815,7 @@
           <t>Scenario →</t>
         </is>
       </c>
-      <c r="B11" s="22">
+      <c r="B11" s="21">
         <f>Assumptions!C4</f>
         <v/>
       </c>
@@ -1835,23 +1831,23 @@
           <t>(Active)</t>
         </is>
       </c>
-      <c r="C12" s="20">
+      <c r="C12" s="19">
         <f>INDEX($C$6:$G$8,MATCH(Assumptions!$C$4,$A$6:$A$8,0),1)</f>
         <v/>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="19">
         <f>INDEX($C$6:$G$8,MATCH(Assumptions!$C$4,$A$6:$A$8,0),2)</f>
         <v/>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="19">
         <f>INDEX($C$6:$G$8,MATCH(Assumptions!$C$4,$A$6:$A$8,0),3)</f>
         <v/>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="19">
         <f>INDEX($C$6:$G$8,MATCH(Assumptions!$C$4,$A$6:$A$8,0),4)</f>
         <v/>
       </c>
-      <c r="G12" s="20">
+      <c r="G12" s="19">
         <f>INDEX($C$6:$G$8,MATCH(Assumptions!$C$4,$A$6:$A$8,0),5)</f>
         <v/>
       </c>
@@ -1885,7 +1881,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>INCOME STATEMENT</t>
         </is>
@@ -1941,28 +1937,28 @@
       <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Total Funds Raised (Active Scenario)</t>
         </is>
       </c>
-      <c r="C6" s="20">
+      <c r="C6" s="19">
         <f>Scenarios!C12</f>
         <v/>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="19">
         <f>Scenarios!D12</f>
         <v/>
       </c>
-      <c r="E6" s="20">
+      <c r="E6" s="19">
         <f>Scenarios!E12</f>
         <v/>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="19">
         <f>Scenarios!F12</f>
         <v/>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="19">
         <f>Scenarios!G12</f>
         <v/>
       </c>
@@ -1973,28 +1969,28 @@
           <t>Upfront Fee Revenue (2% of Funds Raised)</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>→ IS</t>
         </is>
       </c>
-      <c r="C7" s="23">
+      <c r="C7" s="22">
         <f>Assumptions!$C$7*'Income Statement'!C6</f>
         <v/>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="22">
         <f>Assumptions!$C$7*'Income Statement'!D6</f>
         <v/>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="22">
         <f>Assumptions!$C$7*'Income Statement'!E6</f>
         <v/>
       </c>
-      <c r="F7" s="23">
+      <c r="F7" s="22">
         <f>Assumptions!$C$7*'Income Statement'!F6</f>
         <v/>
       </c>
-      <c r="G7" s="23">
+      <c r="G7" s="22">
         <f>Assumptions!$C$7*'Income Statement'!G6</f>
         <v/>
       </c>
@@ -2005,23 +2001,23 @@
           <t>Completion Fee Revenue (0.5% over 3-yr build, straight-line)</t>
         </is>
       </c>
-      <c r="C8" s="23">
+      <c r="C8" s="22">
         <f>(Assumptions!$C$8/Assumptions!$C$9)*('Income Statement'!C6)</f>
         <v/>
       </c>
-      <c r="D8" s="23">
+      <c r="D8" s="22">
         <f>(Assumptions!$C$8/Assumptions!$C$9)*('Income Statement'!C6+D6)</f>
         <v/>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="22">
         <f>(Assumptions!$C$8/Assumptions!$C$9)*('Income Statement'!C6+D6+E6)</f>
         <v/>
       </c>
-      <c r="F8" s="23">
+      <c r="F8" s="22">
         <f>(Assumptions!$C$8/Assumptions!$C$9)*('Income Statement'!D6+E6+F6)</f>
         <v/>
       </c>
-      <c r="G8" s="23">
+      <c r="G8" s="22">
         <f>(Assumptions!$C$8/Assumptions!$C$9)*('Income Statement'!E6+F6+G6)</f>
         <v/>
       </c>
@@ -2032,54 +2028,54 @@
           <t>kWh Revenue (2.12% of Funds, 3-yr lag, cumulative cohorts)</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E9" s="23" t="inlineStr">
+      <c r="E9" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F9" s="23">
+      <c r="F9" s="22">
         <f>Assumptions!$C$11*'Income Statement'!C6</f>
         <v/>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="22">
         <f>Assumptions!$C$11*('Income Statement'!C6+'Income Statement'!D6)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>TOTAL GROSS REVENUE</t>
         </is>
       </c>
-      <c r="B10" s="25" t="n"/>
-      <c r="C10" s="26">
+      <c r="B10" s="24" t="n"/>
+      <c r="C10" s="25">
         <f>SUM('Income Statement'!C7:C9)</f>
         <v/>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="25">
         <f>SUM('Income Statement'!D7:D9)</f>
         <v/>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="25">
         <f>SUM('Income Statement'!E7:E9)</f>
         <v/>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="25">
         <f>SUM('Income Statement'!F7:F9)</f>
         <v/>
       </c>
-      <c r="G10" s="26">
+      <c r="G10" s="25">
         <f>SUM('Income Statement'!G7:G9)</f>
         <v/>
       </c>
@@ -2099,28 +2095,28 @@
       <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Smart Contract Deployment &amp; Audits</t>
         </is>
       </c>
-      <c r="C13" s="20">
+      <c r="C13" s="19">
         <f>Assumptions!C24</f>
         <v/>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="19">
         <f>Assumptions!D24</f>
         <v/>
       </c>
-      <c r="E13" s="20">
+      <c r="E13" s="19">
         <f>Assumptions!E24</f>
         <v/>
       </c>
-      <c r="F13" s="20">
+      <c r="F13" s="19">
         <f>Assumptions!F24</f>
         <v/>
       </c>
-      <c r="G13" s="20">
+      <c r="G13" s="19">
         <f>Assumptions!G24</f>
         <v/>
       </c>
@@ -2131,79 +2127,79 @@
           <t>Hosting &amp; API Costs (1.5% of Gross Revenue)</t>
         </is>
       </c>
-      <c r="C14" s="23">
+      <c r="C14" s="22">
         <f>Assumptions!$C$25*'Income Statement'!C10</f>
         <v/>
       </c>
-      <c r="D14" s="23">
+      <c r="D14" s="22">
         <f>Assumptions!$C$25*'Income Statement'!D10</f>
         <v/>
       </c>
-      <c r="E14" s="23">
+      <c r="E14" s="22">
         <f>Assumptions!$C$25*'Income Statement'!E10</f>
         <v/>
       </c>
-      <c r="F14" s="23">
+      <c r="F14" s="22">
         <f>Assumptions!$C$25*'Income Statement'!F10</f>
         <v/>
       </c>
-      <c r="G14" s="23">
+      <c r="G14" s="22">
         <f>Assumptions!$C$25*'Income Statement'!G10</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>TOTAL COGS</t>
         </is>
       </c>
-      <c r="B15" s="25" t="n"/>
-      <c r="C15" s="26">
+      <c r="B15" s="24" t="n"/>
+      <c r="C15" s="25">
         <f>SUM('Income Statement'!C13:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="26">
+      <c r="D15" s="25">
         <f>SUM('Income Statement'!D13:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="26">
+      <c r="E15" s="25">
         <f>SUM('Income Statement'!E13:E14)</f>
         <v/>
       </c>
-      <c r="F15" s="26">
+      <c r="F15" s="25">
         <f>SUM('Income Statement'!F13:F14)</f>
         <v/>
       </c>
-      <c r="G15" s="26">
+      <c r="G15" s="25">
         <f>SUM('Income Statement'!G13:G14)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="24" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>GROSS PROFIT</t>
         </is>
       </c>
-      <c r="B17" s="25" t="n"/>
-      <c r="C17" s="26">
+      <c r="B17" s="24" t="n"/>
+      <c r="C17" s="25">
         <f>'Income Statement'!C10-'Income Statement'!C15</f>
         <v/>
       </c>
-      <c r="D17" s="26">
+      <c r="D17" s="25">
         <f>'Income Statement'!D10-'Income Statement'!D15</f>
         <v/>
       </c>
-      <c r="E17" s="26">
+      <c r="E17" s="25">
         <f>'Income Statement'!E10-'Income Statement'!E15</f>
         <v/>
       </c>
-      <c r="F17" s="26">
+      <c r="F17" s="25">
         <f>'Income Statement'!F10-'Income Statement'!F15</f>
         <v/>
       </c>
-      <c r="G17" s="26">
+      <c r="G17" s="25">
         <f>'Income Statement'!G10-'Income Statement'!G15</f>
         <v/>
       </c>
@@ -2228,23 +2224,23 @@
           <t>Salaries</t>
         </is>
       </c>
-      <c r="C20" s="20">
+      <c r="C20" s="19">
         <f>Assumptions!$C$28</f>
         <v/>
       </c>
-      <c r="D20" s="23">
+      <c r="D20" s="22">
         <f>Assumptions!D36*'Income Statement'!D10</f>
         <v/>
       </c>
-      <c r="E20" s="23">
+      <c r="E20" s="22">
         <f>Assumptions!E36*'Income Statement'!E10</f>
         <v/>
       </c>
-      <c r="F20" s="23">
+      <c r="F20" s="22">
         <f>Assumptions!F36*'Income Statement'!F10</f>
         <v/>
       </c>
-      <c r="G20" s="23">
+      <c r="G20" s="22">
         <f>Assumptions!G36*'Income Statement'!G10</f>
         <v/>
       </c>
@@ -2255,23 +2251,23 @@
           <t>Marketing &amp; Growth</t>
         </is>
       </c>
-      <c r="C21" s="20">
+      <c r="C21" s="19">
         <f>Assumptions!$C$29</f>
         <v/>
       </c>
-      <c r="D21" s="23">
+      <c r="D21" s="22">
         <f>Assumptions!D37*'Income Statement'!D10</f>
         <v/>
       </c>
-      <c r="E21" s="23">
+      <c r="E21" s="22">
         <f>Assumptions!E37*'Income Statement'!E10</f>
         <v/>
       </c>
-      <c r="F21" s="23">
+      <c r="F21" s="22">
         <f>Assumptions!F37*'Income Statement'!F10</f>
         <v/>
       </c>
-      <c r="G21" s="23">
+      <c r="G21" s="22">
         <f>Assumptions!G37*'Income Statement'!G10</f>
         <v/>
       </c>
@@ -2282,23 +2278,23 @@
           <t>Legal &amp; Regulatory</t>
         </is>
       </c>
-      <c r="C22" s="20">
+      <c r="C22" s="19">
         <f>Assumptions!$C$30</f>
         <v/>
       </c>
-      <c r="D22" s="23">
+      <c r="D22" s="22">
         <f>Assumptions!D38*'Income Statement'!D10</f>
         <v/>
       </c>
-      <c r="E22" s="23">
+      <c r="E22" s="22">
         <f>Assumptions!E38*'Income Statement'!E10</f>
         <v/>
       </c>
-      <c r="F22" s="23">
+      <c r="F22" s="22">
         <f>Assumptions!F38*'Income Statement'!F10</f>
         <v/>
       </c>
-      <c r="G22" s="23">
+      <c r="G22" s="22">
         <f>Assumptions!G38*'Income Statement'!G10</f>
         <v/>
       </c>
@@ -2309,23 +2305,23 @@
           <t>Insurance</t>
         </is>
       </c>
-      <c r="C23" s="20">
+      <c r="C23" s="19">
         <f>Assumptions!$C$31</f>
         <v/>
       </c>
-      <c r="D23" s="23">
+      <c r="D23" s="22">
         <f>Assumptions!D39*'Income Statement'!D10</f>
         <v/>
       </c>
-      <c r="E23" s="23">
+      <c r="E23" s="22">
         <f>Assumptions!E39*'Income Statement'!E10</f>
         <v/>
       </c>
-      <c r="F23" s="23">
+      <c r="F23" s="22">
         <f>Assumptions!F39*'Income Statement'!F10</f>
         <v/>
       </c>
-      <c r="G23" s="23">
+      <c r="G23" s="22">
         <f>Assumptions!G39*'Income Statement'!G10</f>
         <v/>
       </c>
@@ -2336,79 +2332,79 @@
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="C24" s="20">
+      <c r="C24" s="19">
         <f>Assumptions!$C$32</f>
         <v/>
       </c>
-      <c r="D24" s="23">
+      <c r="D24" s="22">
         <f>Assumptions!D40*'Income Statement'!D10</f>
         <v/>
       </c>
-      <c r="E24" s="23">
+      <c r="E24" s="22">
         <f>Assumptions!E40*'Income Statement'!E10</f>
         <v/>
       </c>
-      <c r="F24" s="23">
+      <c r="F24" s="22">
         <f>Assumptions!F40*'Income Statement'!F10</f>
         <v/>
       </c>
-      <c r="G24" s="23">
+      <c r="G24" s="22">
         <f>Assumptions!G40*'Income Statement'!G10</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="23" t="inlineStr">
         <is>
           <t>TOTAL OPERATING EXPENSES</t>
         </is>
       </c>
-      <c r="B25" s="25" t="n"/>
-      <c r="C25" s="26">
+      <c r="B25" s="24" t="n"/>
+      <c r="C25" s="25">
         <f>SUM('Income Statement'!C20:C24)</f>
         <v/>
       </c>
-      <c r="D25" s="26">
+      <c r="D25" s="25">
         <f>SUM('Income Statement'!D20:D24)</f>
         <v/>
       </c>
-      <c r="E25" s="26">
+      <c r="E25" s="25">
         <f>SUM('Income Statement'!E20:E24)</f>
         <v/>
       </c>
-      <c r="F25" s="26">
+      <c r="F25" s="25">
         <f>SUM('Income Statement'!F20:F24)</f>
         <v/>
       </c>
-      <c r="G25" s="26">
+      <c r="G25" s="25">
         <f>SUM('Income Statement'!G20:G24)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="24" t="inlineStr">
+      <c r="A27" s="23" t="inlineStr">
         <is>
           <t>EBIT  (Operating Profit / Loss)</t>
         </is>
       </c>
-      <c r="B27" s="25" t="n"/>
-      <c r="C27" s="26">
+      <c r="B27" s="24" t="n"/>
+      <c r="C27" s="25">
         <f>'Income Statement'!C17-'Income Statement'!C25</f>
         <v/>
       </c>
-      <c r="D27" s="26">
+      <c r="D27" s="25">
         <f>'Income Statement'!D17-'Income Statement'!D25</f>
         <v/>
       </c>
-      <c r="E27" s="26">
+      <c r="E27" s="25">
         <f>'Income Statement'!E17-'Income Statement'!E25</f>
         <v/>
       </c>
-      <c r="F27" s="26">
+      <c r="F27" s="25">
         <f>'Income Statement'!F17-'Income Statement'!F25</f>
         <v/>
       </c>
-      <c r="G27" s="26">
+      <c r="G27" s="25">
         <f>'Income Statement'!G17-'Income Statement'!G25</f>
         <v/>
       </c>
@@ -2433,23 +2429,23 @@
           <t>Prior-Year Tax Loss Balance (b/f)</t>
         </is>
       </c>
-      <c r="C30" s="23">
+      <c r="C30" s="22">
         <f>0</f>
         <v/>
       </c>
-      <c r="D30" s="23">
+      <c r="D30" s="22">
         <f>'Income Statement'!C34</f>
         <v/>
       </c>
-      <c r="E30" s="23">
+      <c r="E30" s="22">
         <f>'Income Statement'!D34</f>
         <v/>
       </c>
-      <c r="F30" s="23">
+      <c r="F30" s="22">
         <f>'Income Statement'!E34</f>
         <v/>
       </c>
-      <c r="G30" s="23">
+      <c r="G30" s="22">
         <f>'Income Statement'!F34</f>
         <v/>
       </c>
@@ -2460,23 +2456,23 @@
           <t>Loss Carry-Forward Applied (limited to £5M p.a. &amp; actual profit)</t>
         </is>
       </c>
-      <c r="C31" s="23">
+      <c r="C31" s="22">
         <f>IF('Income Statement'!C27&gt;0,MIN('Income Statement'!C30,Assumptions!$C$48,'Income Statement'!C27),0)</f>
         <v/>
       </c>
-      <c r="D31" s="23">
+      <c r="D31" s="22">
         <f>IF('Income Statement'!D27&gt;0,MIN('Income Statement'!D30,Assumptions!$C$48,'Income Statement'!D27),0)</f>
         <v/>
       </c>
-      <c r="E31" s="23">
+      <c r="E31" s="22">
         <f>IF('Income Statement'!E27&gt;0,MIN('Income Statement'!E30,Assumptions!$C$48,'Income Statement'!E27),0)</f>
         <v/>
       </c>
-      <c r="F31" s="23">
+      <c r="F31" s="22">
         <f>IF('Income Statement'!F27&gt;0,MIN('Income Statement'!F30,Assumptions!$C$48,'Income Statement'!F27),0)</f>
         <v/>
       </c>
-      <c r="G31" s="23">
+      <c r="G31" s="22">
         <f>IF('Income Statement'!G27&gt;0,MIN('Income Statement'!G30,Assumptions!$C$48,'Income Statement'!G27),0)</f>
         <v/>
       </c>
@@ -2487,23 +2483,23 @@
           <t>Taxable Profit After Loss Relief</t>
         </is>
       </c>
-      <c r="C32" s="23">
+      <c r="C32" s="22">
         <f>MAX('Income Statement'!C27-'Income Statement'!C31,0)</f>
         <v/>
       </c>
-      <c r="D32" s="23">
+      <c r="D32" s="22">
         <f>MAX('Income Statement'!D27-'Income Statement'!D31,0)</f>
         <v/>
       </c>
-      <c r="E32" s="23">
+      <c r="E32" s="22">
         <f>MAX('Income Statement'!E27-'Income Statement'!E31,0)</f>
         <v/>
       </c>
-      <c r="F32" s="23">
+      <c r="F32" s="22">
         <f>MAX('Income Statement'!F27-'Income Statement'!F31,0)</f>
         <v/>
       </c>
-      <c r="G32" s="23">
+      <c r="G32" s="22">
         <f>MAX('Income Statement'!G27-'Income Statement'!G31,0)</f>
         <v/>
       </c>
@@ -2514,23 +2510,23 @@
           <t>Tax Provision (19% / marginal relief / 25%)</t>
         </is>
       </c>
-      <c r="C33" s="23">
+      <c r="C33" s="22">
         <f>IF('Income Statement'!C32&lt;=0,0,IF('Income Statement'!C32&lt;=Assumptions!$C$45,Assumptions!$C$43*'Income Statement'!C32,IF('Income Statement'!C32&lt;=Assumptions!$C$46,Assumptions!$C$44*'Income Statement'!C32-(Assumptions!$C$46-'Income Statement'!C32)*3/200,Assumptions!$C$44*'Income Statement'!C32)))</f>
         <v/>
       </c>
-      <c r="D33" s="23">
+      <c r="D33" s="22">
         <f>IF('Income Statement'!D32&lt;=0,0,IF('Income Statement'!D32&lt;=Assumptions!$C$45,Assumptions!$C$43*'Income Statement'!D32,IF('Income Statement'!D32&lt;=Assumptions!$C$46,Assumptions!$C$44*'Income Statement'!D32-(Assumptions!$C$46-'Income Statement'!D32)*3/200,Assumptions!$C$44*'Income Statement'!D32)))</f>
         <v/>
       </c>
-      <c r="E33" s="23">
+      <c r="E33" s="22">
         <f>IF('Income Statement'!E32&lt;=0,0,IF('Income Statement'!E32&lt;=Assumptions!$C$45,Assumptions!$C$43*'Income Statement'!E32,IF('Income Statement'!E32&lt;=Assumptions!$C$46,Assumptions!$C$44*'Income Statement'!E32-(Assumptions!$C$46-'Income Statement'!E32)*3/200,Assumptions!$C$44*'Income Statement'!E32)))</f>
         <v/>
       </c>
-      <c r="F33" s="23">
+      <c r="F33" s="22">
         <f>IF('Income Statement'!F32&lt;=0,0,IF('Income Statement'!F32&lt;=Assumptions!$C$45,Assumptions!$C$43*'Income Statement'!F32,IF('Income Statement'!F32&lt;=Assumptions!$C$46,Assumptions!$C$44*'Income Statement'!F32-(Assumptions!$C$46-'Income Statement'!F32)*3/200,Assumptions!$C$44*'Income Statement'!F32)))</f>
         <v/>
       </c>
-      <c r="G33" s="23">
+      <c r="G33" s="22">
         <f>IF('Income Statement'!G32&lt;=0,0,IF('Income Statement'!G32&lt;=Assumptions!$C$45,Assumptions!$C$43*'Income Statement'!G32,IF('Income Statement'!G32&lt;=Assumptions!$C$46,Assumptions!$C$44*'Income Statement'!G32-(Assumptions!$C$46-'Income Statement'!G32)*3/200,Assumptions!$C$44*'Income Statement'!G32)))</f>
         <v/>
       </c>
@@ -2541,51 +2537,51 @@
           <t>Closing Tax Loss Balance (carried forward to next year)</t>
         </is>
       </c>
-      <c r="C34" s="23">
+      <c r="C34" s="22">
         <f>MAX(0,'Income Statement'!C30-'Income Statement'!C31)+MAX(0,-'Income Statement'!C27)</f>
         <v/>
       </c>
-      <c r="D34" s="23">
+      <c r="D34" s="22">
         <f>MAX(0,'Income Statement'!D30-'Income Statement'!D31)+MAX(0,-'Income Statement'!D27)</f>
         <v/>
       </c>
-      <c r="E34" s="23">
+      <c r="E34" s="22">
         <f>MAX(0,'Income Statement'!E30-'Income Statement'!E31)+MAX(0,-'Income Statement'!E27)</f>
         <v/>
       </c>
-      <c r="F34" s="23">
+      <c r="F34" s="22">
         <f>MAX(0,'Income Statement'!F30-'Income Statement'!F31)+MAX(0,-'Income Statement'!F27)</f>
         <v/>
       </c>
-      <c r="G34" s="23">
+      <c r="G34" s="22">
         <f>MAX(0,'Income Statement'!G30-'Income Statement'!G31)+MAX(0,-'Income Statement'!G27)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="24" t="inlineStr">
+      <c r="A36" s="23" t="inlineStr">
         <is>
           <t>NET INCOME  (After Tax)</t>
         </is>
       </c>
-      <c r="B36" s="25" t="n"/>
-      <c r="C36" s="27">
+      <c r="B36" s="24" t="n"/>
+      <c r="C36" s="26">
         <f>'Income Statement'!C27-'Income Statement'!C33</f>
         <v/>
       </c>
-      <c r="D36" s="27">
+      <c r="D36" s="26">
         <f>'Income Statement'!D27-'Income Statement'!D33</f>
         <v/>
       </c>
-      <c r="E36" s="27">
+      <c r="E36" s="26">
         <f>'Income Statement'!E27-'Income Statement'!E33</f>
         <v/>
       </c>
-      <c r="F36" s="27">
+      <c r="F36" s="26">
         <f>'Income Statement'!F27-'Income Statement'!F33</f>
         <v/>
       </c>
-      <c r="G36" s="27">
+      <c r="G36" s="26">
         <f>'Income Statement'!G27-'Income Statement'!G33</f>
         <v/>
       </c>
@@ -2617,7 +2613,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>BALANCE SHEET</t>
         </is>
@@ -2630,14 +2626,14 @@
       <c r="G1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="27" t="inlineStr">
         <is>
           <t>All figures in GBP (£)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="29" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>Year →</t>
         </is>
@@ -2673,28 +2669,28 @@
       <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Cash &amp; Cash Equivalents</t>
         </is>
       </c>
-      <c r="C6" s="20">
+      <c r="C6" s="19">
         <f>'Cash Flow'!C23</f>
         <v/>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="19">
         <f>'Cash Flow'!D23</f>
         <v/>
       </c>
-      <c r="E6" s="20">
+      <c r="E6" s="19">
         <f>'Cash Flow'!E23</f>
         <v/>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="19">
         <f>'Cash Flow'!F23</f>
         <v/>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="19">
         <f>'Cash Flow'!G23</f>
         <v/>
       </c>
@@ -2705,79 +2701,79 @@
           <t>Accounts Receivable  (Revenue × DSO / 365)</t>
         </is>
       </c>
-      <c r="C7" s="23">
+      <c r="C7" s="22">
         <f>'Income Statement'!C10*Assumptions!$C$55/365</f>
         <v/>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="22">
         <f>'Income Statement'!D10*Assumptions!$C$55/365</f>
         <v/>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="22">
         <f>'Income Statement'!E10*Assumptions!$C$55/365</f>
         <v/>
       </c>
-      <c r="F7" s="23">
+      <c r="F7" s="22">
         <f>'Income Statement'!F10*Assumptions!$C$55/365</f>
         <v/>
       </c>
-      <c r="G7" s="23">
+      <c r="G7" s="22">
         <f>'Income Statement'!G10*Assumptions!$C$55/365</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>TOTAL CURRENT ASSETS</t>
         </is>
       </c>
-      <c r="B8" s="25" t="n"/>
-      <c r="C8" s="26">
+      <c r="B8" s="24" t="n"/>
+      <c r="C8" s="25">
         <f>SUM('Balance Sheet'!C6:C7)</f>
         <v/>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="25">
         <f>SUM('Balance Sheet'!D6:D7)</f>
         <v/>
       </c>
-      <c r="E8" s="26">
+      <c r="E8" s="25">
         <f>SUM('Balance Sheet'!E6:E7)</f>
         <v/>
       </c>
-      <c r="F8" s="26">
+      <c r="F8" s="25">
         <f>SUM('Balance Sheet'!F6:F7)</f>
         <v/>
       </c>
-      <c r="G8" s="26">
+      <c r="G8" s="25">
         <f>SUM('Balance Sheet'!G6:G7)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>TOTAL ASSETS</t>
         </is>
       </c>
-      <c r="B9" s="25" t="n"/>
-      <c r="C9" s="30">
+      <c r="B9" s="24" t="n"/>
+      <c r="C9" s="29">
         <f>'Balance Sheet'!C8</f>
         <v/>
       </c>
-      <c r="D9" s="30">
+      <c r="D9" s="29">
         <f>'Balance Sheet'!D8</f>
         <v/>
       </c>
-      <c r="E9" s="30">
+      <c r="E9" s="29">
         <f>'Balance Sheet'!E8</f>
         <v/>
       </c>
-      <c r="F9" s="30">
+      <c r="F9" s="29">
         <f>'Balance Sheet'!F8</f>
         <v/>
       </c>
-      <c r="G9" s="30">
+      <c r="G9" s="29">
         <f>'Balance Sheet'!G8</f>
         <v/>
       </c>
@@ -2802,23 +2798,23 @@
           <t>Accounts Payable  ((COGS + OpEx) × DPO / 365)</t>
         </is>
       </c>
-      <c r="C12" s="23">
+      <c r="C12" s="22">
         <f>('Income Statement'!C15+'Income Statement'!C25)*Assumptions!$C$56/365</f>
         <v/>
       </c>
-      <c r="D12" s="23">
+      <c r="D12" s="22">
         <f>('Income Statement'!D15+'Income Statement'!D25)*Assumptions!$C$56/365</f>
         <v/>
       </c>
-      <c r="E12" s="23">
+      <c r="E12" s="22">
         <f>('Income Statement'!E15+'Income Statement'!E25)*Assumptions!$C$56/365</f>
         <v/>
       </c>
-      <c r="F12" s="23">
+      <c r="F12" s="22">
         <f>('Income Statement'!F15+'Income Statement'!F25)*Assumptions!$C$56/365</f>
         <v/>
       </c>
-      <c r="G12" s="23">
+      <c r="G12" s="22">
         <f>('Income Statement'!G15+'Income Statement'!G25)*Assumptions!$C$56/365</f>
         <v/>
       </c>
@@ -2829,79 +2825,79 @@
           <t>Corporation Tax Payable  (current year provision, paid next year)</t>
         </is>
       </c>
-      <c r="C13" s="23">
+      <c r="C13" s="22">
         <f>'Income Statement'!C33</f>
         <v/>
       </c>
-      <c r="D13" s="23">
+      <c r="D13" s="22">
         <f>'Income Statement'!D33</f>
         <v/>
       </c>
-      <c r="E13" s="23">
+      <c r="E13" s="22">
         <f>'Income Statement'!E33</f>
         <v/>
       </c>
-      <c r="F13" s="23">
+      <c r="F13" s="22">
         <f>'Income Statement'!F33</f>
         <v/>
       </c>
-      <c r="G13" s="23">
+      <c r="G13" s="22">
         <f>'Income Statement'!G33</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>TOTAL CURRENT LIABILITIES</t>
         </is>
       </c>
-      <c r="B14" s="25" t="n"/>
-      <c r="C14" s="26">
+      <c r="B14" s="24" t="n"/>
+      <c r="C14" s="25">
         <f>SUM('Balance Sheet'!C12:C13)</f>
         <v/>
       </c>
-      <c r="D14" s="26">
+      <c r="D14" s="25">
         <f>SUM('Balance Sheet'!D12:D13)</f>
         <v/>
       </c>
-      <c r="E14" s="26">
+      <c r="E14" s="25">
         <f>SUM('Balance Sheet'!E12:E13)</f>
         <v/>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="25">
         <f>SUM('Balance Sheet'!F12:F13)</f>
         <v/>
       </c>
-      <c r="G14" s="26">
+      <c r="G14" s="25">
         <f>SUM('Balance Sheet'!G12:G13)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>TOTAL LIABILITIES</t>
         </is>
       </c>
-      <c r="B15" s="25" t="n"/>
-      <c r="C15" s="30">
+      <c r="B15" s="24" t="n"/>
+      <c r="C15" s="29">
         <f>'Balance Sheet'!C14</f>
         <v/>
       </c>
-      <c r="D15" s="30">
+      <c r="D15" s="29">
         <f>'Balance Sheet'!D14</f>
         <v/>
       </c>
-      <c r="E15" s="30">
+      <c r="E15" s="29">
         <f>'Balance Sheet'!E14</f>
         <v/>
       </c>
-      <c r="F15" s="30">
+      <c r="F15" s="29">
         <f>'Balance Sheet'!F14</f>
         <v/>
       </c>
-      <c r="G15" s="30">
+      <c r="G15" s="29">
         <f>'Balance Sheet'!G14</f>
         <v/>
       </c>
@@ -2921,28 +2917,28 @@
       <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>Share Capital  (cumulative equity raises to date)</t>
         </is>
       </c>
-      <c r="C18" s="20">
+      <c r="C18" s="19">
         <f>Assumptions!C52</f>
         <v/>
       </c>
-      <c r="D18" s="20">
+      <c r="D18" s="19">
         <f>'Balance Sheet'!C18+Assumptions!D52</f>
         <v/>
       </c>
-      <c r="E18" s="20">
+      <c r="E18" s="19">
         <f>'Balance Sheet'!D18+Assumptions!E52</f>
         <v/>
       </c>
-      <c r="F18" s="20">
+      <c r="F18" s="19">
         <f>'Balance Sheet'!E18+Assumptions!F52</f>
         <v/>
       </c>
-      <c r="G18" s="20">
+      <c r="G18" s="19">
         <f>'Balance Sheet'!F18+Assumptions!G52</f>
         <v/>
       </c>
@@ -2953,51 +2949,51 @@
           <t>Retained Earnings  (cumulative net income)</t>
         </is>
       </c>
-      <c r="C19" s="23">
+      <c r="C19" s="22">
         <f>'Income Statement'!C36</f>
         <v/>
       </c>
-      <c r="D19" s="23">
+      <c r="D19" s="22">
         <f>'Balance Sheet'!C19+'Income Statement'!D36</f>
         <v/>
       </c>
-      <c r="E19" s="23">
+      <c r="E19" s="22">
         <f>'Balance Sheet'!D19+'Income Statement'!E36</f>
         <v/>
       </c>
-      <c r="F19" s="23">
+      <c r="F19" s="22">
         <f>'Balance Sheet'!E19+'Income Statement'!F36</f>
         <v/>
       </c>
-      <c r="G19" s="23">
+      <c r="G19" s="22">
         <f>'Balance Sheet'!F19+'Income Statement'!G36</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="A20" s="23" t="inlineStr">
         <is>
           <t>TOTAL EQUITY</t>
         </is>
       </c>
-      <c r="B20" s="25" t="n"/>
-      <c r="C20" s="30">
+      <c r="B20" s="24" t="n"/>
+      <c r="C20" s="29">
         <f>SUM('Balance Sheet'!C18:C19)</f>
         <v/>
       </c>
-      <c r="D20" s="30">
+      <c r="D20" s="29">
         <f>SUM('Balance Sheet'!D18:D19)</f>
         <v/>
       </c>
-      <c r="E20" s="30">
+      <c r="E20" s="29">
         <f>SUM('Balance Sheet'!E18:E19)</f>
         <v/>
       </c>
-      <c r="F20" s="30">
+      <c r="F20" s="29">
         <f>SUM('Balance Sheet'!F18:F19)</f>
         <v/>
       </c>
-      <c r="G20" s="30">
+      <c r="G20" s="29">
         <f>SUM('Balance Sheet'!G18:G19)</f>
         <v/>
       </c>
@@ -3009,23 +3005,23 @@
         </is>
       </c>
       <c r="B22" s="2" t="n"/>
-      <c r="C22" s="31">
+      <c r="C22" s="30">
         <f>'Balance Sheet'!C9-'Balance Sheet'!C15-'Balance Sheet'!C20</f>
         <v/>
       </c>
-      <c r="D22" s="31">
+      <c r="D22" s="30">
         <f>'Balance Sheet'!D9-'Balance Sheet'!D15-'Balance Sheet'!D20</f>
         <v/>
       </c>
-      <c r="E22" s="31">
+      <c r="E22" s="30">
         <f>'Balance Sheet'!E9-'Balance Sheet'!E15-'Balance Sheet'!E20</f>
         <v/>
       </c>
-      <c r="F22" s="31">
+      <c r="F22" s="30">
         <f>'Balance Sheet'!F9-'Balance Sheet'!F15-'Balance Sheet'!F20</f>
         <v/>
       </c>
-      <c r="G22" s="31">
+      <c r="G22" s="30">
         <f>'Balance Sheet'!G9-'Balance Sheet'!G15-'Balance Sheet'!G20</f>
         <v/>
       </c>
@@ -3058,7 +3054,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>CASH FLOW STATEMENT  (Indirect Method)</t>
         </is>
@@ -3071,14 +3067,14 @@
       <c r="G1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="28" t="inlineStr">
+      <c r="A2" s="27" t="inlineStr">
         <is>
           <t>All figures in GBP (£)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="29" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>Year →</t>
         </is>
@@ -3114,28 +3110,28 @@
       <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Net Income (after tax)</t>
         </is>
       </c>
-      <c r="C6" s="20">
+      <c r="C6" s="19">
         <f>'Income Statement'!C36</f>
         <v/>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="19">
         <f>'Income Statement'!D36</f>
         <v/>
       </c>
-      <c r="E6" s="20">
+      <c r="E6" s="19">
         <f>'Income Statement'!E36</f>
         <v/>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="19">
         <f>'Income Statement'!F36</f>
         <v/>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="19">
         <f>'Income Statement'!G36</f>
         <v/>
       </c>
@@ -3146,23 +3142,23 @@
           <t>Change in Accounts Receivable  (increase = cash outflow)</t>
         </is>
       </c>
-      <c r="C7" s="23">
+      <c r="C7" s="22">
         <f>-('Balance Sheet'!C7-0)</f>
         <v/>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="22">
         <f>-('Balance Sheet'!D7-'Balance Sheet'!C7)</f>
         <v/>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="22">
         <f>-('Balance Sheet'!E7-'Balance Sheet'!D7)</f>
         <v/>
       </c>
-      <c r="F7" s="23">
+      <c r="F7" s="22">
         <f>-('Balance Sheet'!F7-'Balance Sheet'!E7)</f>
         <v/>
       </c>
-      <c r="G7" s="23">
+      <c r="G7" s="22">
         <f>-('Balance Sheet'!G7-'Balance Sheet'!F7)</f>
         <v/>
       </c>
@@ -3173,23 +3169,23 @@
           <t>Change in Accounts Payable  (increase = cash inflow)</t>
         </is>
       </c>
-      <c r="C8" s="23">
+      <c r="C8" s="22">
         <f>'Balance Sheet'!C12-0</f>
         <v/>
       </c>
-      <c r="D8" s="23">
+      <c r="D8" s="22">
         <f>'Balance Sheet'!D12-'Balance Sheet'!C12</f>
         <v/>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="22">
         <f>'Balance Sheet'!E12-'Balance Sheet'!D12</f>
         <v/>
       </c>
-      <c r="F8" s="23">
+      <c r="F8" s="22">
         <f>'Balance Sheet'!F12-'Balance Sheet'!E12</f>
         <v/>
       </c>
-      <c r="G8" s="23">
+      <c r="G8" s="22">
         <f>'Balance Sheet'!G12-'Balance Sheet'!F12</f>
         <v/>
       </c>
@@ -3200,51 +3196,51 @@
           <t>Change in Corporation Tax Payable  (current provision − prior paid)</t>
         </is>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="22">
         <f>'Balance Sheet'!C13-0</f>
         <v/>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="22">
         <f>'Balance Sheet'!D13-'Balance Sheet'!C13</f>
         <v/>
       </c>
-      <c r="E9" s="23">
+      <c r="E9" s="22">
         <f>'Balance Sheet'!E13-'Balance Sheet'!D13</f>
         <v/>
       </c>
-      <c r="F9" s="23">
+      <c r="F9" s="22">
         <f>'Balance Sheet'!F13-'Balance Sheet'!E13</f>
         <v/>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="22">
         <f>'Balance Sheet'!G13-'Balance Sheet'!F13</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>NET CASH FROM OPERATIONS</t>
         </is>
       </c>
-      <c r="B10" s="25" t="n"/>
-      <c r="C10" s="26">
+      <c r="B10" s="24" t="n"/>
+      <c r="C10" s="25">
         <f>SUM('Cash Flow'!C6:C9)</f>
         <v/>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="25">
         <f>SUM('Cash Flow'!D6:D9)</f>
         <v/>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="25">
         <f>SUM('Cash Flow'!E6:E9)</f>
         <v/>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="25">
         <f>SUM('Cash Flow'!F6:F9)</f>
         <v/>
       </c>
-      <c r="G10" s="26">
+      <c r="G10" s="25">
         <f>SUM('Cash Flow'!G6:G9)</f>
         <v/>
       </c>
@@ -3264,56 +3260,56 @@
       <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Capital Expenditure / CapEx  (asset-light — £0)</t>
         </is>
       </c>
-      <c r="C13" s="20">
+      <c r="C13" s="19">
         <f>-Assumptions!$C$62</f>
         <v/>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="19">
         <f>-Assumptions!$C$62</f>
         <v/>
       </c>
-      <c r="E13" s="20">
+      <c r="E13" s="19">
         <f>-Assumptions!$C$62</f>
         <v/>
       </c>
-      <c r="F13" s="20">
+      <c r="F13" s="19">
         <f>-Assumptions!$C$62</f>
         <v/>
       </c>
-      <c r="G13" s="20">
+      <c r="G13" s="19">
         <f>-Assumptions!$C$62</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>NET CASH FROM INVESTING</t>
         </is>
       </c>
-      <c r="B14" s="25" t="n"/>
-      <c r="C14" s="26">
+      <c r="B14" s="24" t="n"/>
+      <c r="C14" s="25">
         <f>'Cash Flow'!C13</f>
         <v/>
       </c>
-      <c r="D14" s="26">
+      <c r="D14" s="25">
         <f>'Cash Flow'!D13</f>
         <v/>
       </c>
-      <c r="E14" s="26">
+      <c r="E14" s="25">
         <f>'Cash Flow'!E13</f>
         <v/>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="25">
         <f>'Cash Flow'!F13</f>
         <v/>
       </c>
-      <c r="G14" s="26">
+      <c r="G14" s="25">
         <f>'Cash Flow'!G13</f>
         <v/>
       </c>
@@ -3333,56 +3329,56 @@
       <c r="H16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>Equity Raised  (per Assumptions)</t>
         </is>
       </c>
-      <c r="C17" s="20">
+      <c r="C17" s="19">
         <f>Assumptions!C52</f>
         <v/>
       </c>
-      <c r="D17" s="20">
+      <c r="D17" s="19">
         <f>Assumptions!D52</f>
         <v/>
       </c>
-      <c r="E17" s="20">
+      <c r="E17" s="19">
         <f>Assumptions!E52</f>
         <v/>
       </c>
-      <c r="F17" s="20">
+      <c r="F17" s="19">
         <f>Assumptions!F52</f>
         <v/>
       </c>
-      <c r="G17" s="20">
+      <c r="G17" s="19">
         <f>Assumptions!G52</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>NET CASH FROM FINANCING</t>
         </is>
       </c>
-      <c r="B18" s="25" t="n"/>
-      <c r="C18" s="26">
+      <c r="B18" s="24" t="n"/>
+      <c r="C18" s="25">
         <f>'Cash Flow'!C17</f>
         <v/>
       </c>
-      <c r="D18" s="26">
+      <c r="D18" s="25">
         <f>'Cash Flow'!D17</f>
         <v/>
       </c>
-      <c r="E18" s="26">
+      <c r="E18" s="25">
         <f>'Cash Flow'!E17</f>
         <v/>
       </c>
-      <c r="F18" s="26">
+      <c r="F18" s="25">
         <f>'Cash Flow'!F17</f>
         <v/>
       </c>
-      <c r="G18" s="26">
+      <c r="G18" s="25">
         <f>'Cash Flow'!G17</f>
         <v/>
       </c>
@@ -3407,23 +3403,23 @@
           <t>Net Change in Cash</t>
         </is>
       </c>
-      <c r="C21" s="23">
+      <c r="C21" s="22">
         <f>'Cash Flow'!C10+'Cash Flow'!C14+'Cash Flow'!C18</f>
         <v/>
       </c>
-      <c r="D21" s="23">
+      <c r="D21" s="22">
         <f>'Cash Flow'!D10+'Cash Flow'!D14+'Cash Flow'!D18</f>
         <v/>
       </c>
-      <c r="E21" s="23">
+      <c r="E21" s="22">
         <f>'Cash Flow'!E10+'Cash Flow'!E14+'Cash Flow'!E18</f>
         <v/>
       </c>
-      <c r="F21" s="23">
+      <c r="F21" s="22">
         <f>'Cash Flow'!F10+'Cash Flow'!F14+'Cash Flow'!F18</f>
         <v/>
       </c>
-      <c r="G21" s="23">
+      <c r="G21" s="22">
         <f>'Cash Flow'!G10+'Cash Flow'!G14+'Cash Flow'!G18</f>
         <v/>
       </c>
@@ -3434,51 +3430,51 @@
           <t>Opening Cash</t>
         </is>
       </c>
-      <c r="C22" s="20">
+      <c r="C22" s="19">
         <f>Assumptions!$C$59</f>
         <v/>
       </c>
-      <c r="D22" s="23">
+      <c r="D22" s="22">
         <f>'Cash Flow'!C23</f>
         <v/>
       </c>
-      <c r="E22" s="23">
+      <c r="E22" s="22">
         <f>'Cash Flow'!D23</f>
         <v/>
       </c>
-      <c r="F22" s="23">
+      <c r="F22" s="22">
         <f>'Cash Flow'!E23</f>
         <v/>
       </c>
-      <c r="G22" s="23">
+      <c r="G22" s="22">
         <f>'Cash Flow'!F23</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="24" t="inlineStr">
+      <c r="A23" s="23" t="inlineStr">
         <is>
           <t>CLOSING CASH  (= Balance Sheet: Cash &amp; Cash Equivalents)</t>
         </is>
       </c>
-      <c r="B23" s="25" t="n"/>
-      <c r="C23" s="27">
+      <c r="B23" s="24" t="n"/>
+      <c r="C23" s="26">
         <f>'Cash Flow'!C21+'Cash Flow'!C22</f>
         <v/>
       </c>
-      <c r="D23" s="27">
+      <c r="D23" s="26">
         <f>'Cash Flow'!D21+'Cash Flow'!D22</f>
         <v/>
       </c>
-      <c r="E23" s="27">
+      <c r="E23" s="26">
         <f>'Cash Flow'!E21+'Cash Flow'!E22</f>
         <v/>
       </c>
-      <c r="F23" s="27">
+      <c r="F23" s="26">
         <f>'Cash Flow'!F21+'Cash Flow'!F22</f>
         <v/>
       </c>
-      <c r="G23" s="27">
+      <c r="G23" s="26">
         <f>'Cash Flow'!G21+'Cash Flow'!G22</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add Valuation and Cap Table sheets to financial model
Agent-Logs-Url: https://github.com/DejAmour/Joule-Financial-Model/sessions/acd1d82e-a489-4fd4-b1f8-9ea7047a5f63

Co-authored-by: DejAmour <159169578+DejAmour@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/financial_model.xlsx
+++ b/financial_model.xlsx
@@ -12,6 +12,8 @@
     <sheet name="Income Statement" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Balance Sheet" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Cash Flow" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Valuation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cap Table" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Assumptions'!$1:$3</definedName>
@@ -19,6 +21,8 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Income Statement'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Balance Sheet'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Cash Flow'!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Valuation'!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Cap Table'!$1:$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,11 +30,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="£#,##0.00"/>
     <numFmt numFmtId="166" formatCode="£#,##0"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="0&quot;x&quot;"/>
+    <numFmt numFmtId="169" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="170" formatCode="0.0000"/>
+    <numFmt numFmtId="171" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="172" formatCode="0.0000%"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -87,7 +96,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -107,6 +116,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -149,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -225,6 +239,72 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -483,6 +563,115 @@
 − Prior year tax provision  (now settled in cash, 9-month lag)
 Net = change in Tax Payable balance.
 This ensures the Balance Sheet balances correctly.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Joule Model</author>
+  </authors>
+  <commentList>
+    <comment ref="C10" authorId="0" shapeId="0">
+      <text>
+        <t>Tiered discount rates (FAST VC convention):
+  Y1-3:  50% (highest risk — early stage)
+  Y4-6:  35% (growth stage)
+  Y7-10: 25% (more mature, lower risk)
+Discount is compounded through each tier cumulatively.</t>
+      </text>
+    </comment>
+    <comment ref="D18" authorId="0" shapeId="0">
+      <text>
+        <t>Years 1-5: linked directly to 'Income Statement'!C10:G10 (Total Gross Revenue).
+Years 6-10: prior year revenue × (1 + Revenue CAGR Y5-Y10) = 60% growth.</t>
+      </text>
+    </comment>
+    <comment ref="A26" authorId="0" shapeId="0">
+      <text>
+        <t>Cash logic by year:
+  Exit year (5): linked to 'Balance Sheet'!G6 (closing cash 2030)
+  Years 6-10: 2% of net revenue (proxy for cash balance)
+  All other years: £0</t>
+      </text>
+    </comment>
+    <comment ref="A27" authorId="0" shapeId="0">
+      <text>
+        <t>Equity Value calculation:
+  Years 1-5 (up to exit): EV + Financial Debt + Cash
+  Years 6-10 (post-exit): prior year Equity Value × (1 + Equity Growth Rate)</t>
+      </text>
+    </comment>
+    <comment ref="A28" authorId="0" shapeId="0">
+      <text>
+        <t>Tiered discount rate:
+  Years 1-3:  50% (C10)
+  Years 4-6:  35% (C11)
+  Years 7-10: 25% (C12)</t>
+      </text>
+    </comment>
+    <comment ref="A31" authorId="0" shapeId="0">
+      <text>
+        <t>Present Value uses compound tiered discounting:
+  PV = Equity Value / ((1+r_y1_3)^y1_3_yrs × (1+r_y3_6)^y3_6_yrs × (1+r_y6_10)^y6_10_yrs)
+  Only calculated from exit year (5) onwards.
+  y1_3_yrs = MIN(n,3)
+  y3_6_yrs = MAX(0, MIN(n,6)-3)
+  y6_10_yrs = MAX(0, n-6)</t>
+      </text>
+    </comment>
+    <comment ref="C35" authorId="0" shapeId="0">
+      <text>
+        <t>Linked to Cap Table!C9 — Pre-seed T1 ownership % granted at round.</t>
+      </text>
+    </comment>
+    <comment ref="C36" authorId="0" shapeId="0">
+      <text>
+        <t>Dilution = Pre-seed T1 final ownership % (Section D, row 30) minus initial stake (Section B, row 9).
+Negative value = dilution from subsequent funding rounds.</t>
+      </text>
+    </comment>
+    <comment ref="C40" authorId="0" shapeId="0">
+      <text>
+        <t>IRR uses Excel's built-in IRR() function on the investor cash flow series.
+Cash flows: Year 0 = -Investment; Years 1-4 = 0; Year 5 = Exit Proceeds; Years 6-10 = 0.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Joule Model</author>
+  </authors>
+  <commentList>
+    <comment ref="J2" authorId="0" shapeId="0">
+      <text>
+        <t>GBP/USD FX rate used for $ conversions.
+Hardcoded fallback = 0.7577. Update cell directly to refresh $ columns.</t>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>Founder shares: 1,000,000 (from Assumptions)</t>
+      </text>
+    </comment>
+    <comment ref="D8" authorId="0" shapeId="0">
+      <text>
+        <t>Shares Issued formula (correct cumulative dilution):
+  new_shares = cumulative_shares / (1 - ownership_pct) - cumulative_shares
+  Uses running total of ALL shares outstanding before this round.
+  This ensures investors receive exactly their target post-round ownership %.</t>
+      </text>
+    </comment>
+    <comment ref="C36" authorId="0" shapeId="0">
+      <text>
+        <t>Should equal 100%. If not, check shares-issued formulas.</t>
       </text>
     </comment>
   </commentList>
@@ -3484,4 +3673,1921 @@
   <pageSetup orientation="landscape" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C65911"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:N47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>VALUATION MODEL — VC METHOD</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>All figures in GBP (£) unless stated</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>A. VALUATION ASSUMPTIONS</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Valuation Date</t>
+        </is>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>2025-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Exit Year</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>EV / Revenue Multiple</t>
+        </is>
+      </c>
+      <c r="C7" s="32" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Financial Debt at Exit (£)</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Cash at Exit (£)  [→ Balance Sheet G6]</t>
+        </is>
+      </c>
+      <c r="C9" s="33">
+        <f>'Balance Sheet'!G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Required Return Y1-3</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Required Return Y4-6</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Required Return Y7-10</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Revenue CAGR Y5-Y10</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Equity Growth Rate Y5-Y10</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Forecast Year →</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J16" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="K16" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="L16" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="M16" s="9" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>B. REVENUE PROJECTIONS  (£)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n"/>
+      <c r="M17" s="2" t="n"/>
+      <c r="N17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Net Revenue (Total Gross Revenue)</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="19">
+        <f>'Income Statement'!C10</f>
+        <v/>
+      </c>
+      <c r="E18" s="19">
+        <f>'Income Statement'!D10</f>
+        <v/>
+      </c>
+      <c r="F18" s="19">
+        <f>'Income Statement'!E10</f>
+        <v/>
+      </c>
+      <c r="G18" s="19">
+        <f>'Income Statement'!F10</f>
+        <v/>
+      </c>
+      <c r="H18" s="19">
+        <f>'Income Statement'!G10</f>
+        <v/>
+      </c>
+      <c r="I18" s="22">
+        <f>H18*(1+$C$13)</f>
+        <v/>
+      </c>
+      <c r="J18" s="22">
+        <f>I18*(1+$C$13)</f>
+        <v/>
+      </c>
+      <c r="K18" s="22">
+        <f>J18*(1+$C$13)</f>
+        <v/>
+      </c>
+      <c r="L18" s="22">
+        <f>K18*(1+$C$13)</f>
+        <v/>
+      </c>
+      <c r="M18" s="22">
+        <f>L18*(1+$C$13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>C. VC VALUATION TABLE</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n"/>
+      <c r="M20" s="2" t="n"/>
+      <c r="N20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Forecast Year</t>
+        </is>
+      </c>
+      <c r="C21" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="H21" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="I21" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="J21" s="34" t="n">
+        <v>7</v>
+      </c>
+      <c r="K21" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="L21" s="34" t="n">
+        <v>9</v>
+      </c>
+      <c r="M21" s="34" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Cash Flow Date</t>
+        </is>
+      </c>
+      <c r="C22" s="35">
+        <f>$C$5</f>
+        <v/>
+      </c>
+      <c r="D22" s="35">
+        <f>EDATE(C22,12)</f>
+        <v/>
+      </c>
+      <c r="E22" s="35">
+        <f>EDATE(D22,12)</f>
+        <v/>
+      </c>
+      <c r="F22" s="35">
+        <f>EDATE(E22,12)</f>
+        <v/>
+      </c>
+      <c r="G22" s="35">
+        <f>EDATE(F22,12)</f>
+        <v/>
+      </c>
+      <c r="H22" s="35">
+        <f>EDATE(G22,12)</f>
+        <v/>
+      </c>
+      <c r="I22" s="35">
+        <f>EDATE(H22,12)</f>
+        <v/>
+      </c>
+      <c r="J22" s="35">
+        <f>EDATE(I22,12)</f>
+        <v/>
+      </c>
+      <c r="K22" s="35">
+        <f>EDATE(J22,12)</f>
+        <v/>
+      </c>
+      <c r="L22" s="35">
+        <f>EDATE(K22,12)</f>
+        <v/>
+      </c>
+      <c r="M22" s="35">
+        <f>EDATE(L22,12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Net Revenue (£)</t>
+        </is>
+      </c>
+      <c r="C23" s="22">
+        <f>C18</f>
+        <v/>
+      </c>
+      <c r="D23" s="22">
+        <f>D18</f>
+        <v/>
+      </c>
+      <c r="E23" s="22">
+        <f>E18</f>
+        <v/>
+      </c>
+      <c r="F23" s="22">
+        <f>F18</f>
+        <v/>
+      </c>
+      <c r="G23" s="22">
+        <f>G18</f>
+        <v/>
+      </c>
+      <c r="H23" s="22">
+        <f>H18</f>
+        <v/>
+      </c>
+      <c r="I23" s="22">
+        <f>I18</f>
+        <v/>
+      </c>
+      <c r="J23" s="22">
+        <f>J18</f>
+        <v/>
+      </c>
+      <c r="K23" s="22">
+        <f>K18</f>
+        <v/>
+      </c>
+      <c r="L23" s="22">
+        <f>L18</f>
+        <v/>
+      </c>
+      <c r="M23" s="22">
+        <f>M18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Enterprise Value  (EV = Revenue × Multiple)</t>
+        </is>
+      </c>
+      <c r="C24" s="22">
+        <f>C23*$C$7</f>
+        <v/>
+      </c>
+      <c r="D24" s="22">
+        <f>D23*$C$7</f>
+        <v/>
+      </c>
+      <c r="E24" s="22">
+        <f>E23*$C$7</f>
+        <v/>
+      </c>
+      <c r="F24" s="22">
+        <f>F23*$C$7</f>
+        <v/>
+      </c>
+      <c r="G24" s="22">
+        <f>G23*$C$7</f>
+        <v/>
+      </c>
+      <c r="H24" s="22">
+        <f>H23*$C$7</f>
+        <v/>
+      </c>
+      <c r="I24" s="22">
+        <f>I23*$C$7</f>
+        <v/>
+      </c>
+      <c r="J24" s="22">
+        <f>J23*$C$7</f>
+        <v/>
+      </c>
+      <c r="K24" s="22">
+        <f>K23*$C$7</f>
+        <v/>
+      </c>
+      <c r="L24" s="22">
+        <f>L23*$C$7</f>
+        <v/>
+      </c>
+      <c r="M24" s="22">
+        <f>M23*$C$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Financial Debt at Exit (£)</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="22">
+        <f>IF(D21=$C$6,-$C$8,0)</f>
+        <v/>
+      </c>
+      <c r="E25" s="22">
+        <f>IF(E21=$C$6,-$C$8,0)</f>
+        <v/>
+      </c>
+      <c r="F25" s="22">
+        <f>IF(F21=$C$6,-$C$8,0)</f>
+        <v/>
+      </c>
+      <c r="G25" s="22">
+        <f>IF(G21=$C$6,-$C$8,0)</f>
+        <v/>
+      </c>
+      <c r="H25" s="22">
+        <f>IF(H21=$C$6,-$C$8,0)</f>
+        <v/>
+      </c>
+      <c r="I25" s="22">
+        <f>IF(I21=$C$6,-$C$8,0)</f>
+        <v/>
+      </c>
+      <c r="J25" s="22">
+        <f>IF(J21=$C$6,-$C$8,0)</f>
+        <v/>
+      </c>
+      <c r="K25" s="22">
+        <f>IF(K21=$C$6,-$C$8,0)</f>
+        <v/>
+      </c>
+      <c r="L25" s="22">
+        <f>IF(L21=$C$6,-$C$8,0)</f>
+        <v/>
+      </c>
+      <c r="M25" s="22">
+        <f>IF(M21=$C$6,-$C$8,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Cash at Exit / 2% of Revenue (£)</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="22">
+        <f>IF(D21=$C$6,$C$9,IF(D21&gt;$C$6,D23*0.02,0))</f>
+        <v/>
+      </c>
+      <c r="E26" s="22">
+        <f>IF(E21=$C$6,$C$9,IF(E21&gt;$C$6,E23*0.02,0))</f>
+        <v/>
+      </c>
+      <c r="F26" s="22">
+        <f>IF(F21=$C$6,$C$9,IF(F21&gt;$C$6,F23*0.02,0))</f>
+        <v/>
+      </c>
+      <c r="G26" s="22">
+        <f>IF(G21=$C$6,$C$9,IF(G21&gt;$C$6,G23*0.02,0))</f>
+        <v/>
+      </c>
+      <c r="H26" s="19">
+        <f>IF(H21=$C$6,$C$9,IF(H21&gt;$C$6,H23*0.02,0))</f>
+        <v/>
+      </c>
+      <c r="I26" s="22">
+        <f>IF(I21=$C$6,$C$9,IF(I21&gt;$C$6,I23*0.02,0))</f>
+        <v/>
+      </c>
+      <c r="J26" s="22">
+        <f>IF(J21=$C$6,$C$9,IF(J21&gt;$C$6,J23*0.02,0))</f>
+        <v/>
+      </c>
+      <c r="K26" s="22">
+        <f>IF(K21=$C$6,$C$9,IF(K21&gt;$C$6,K23*0.02,0))</f>
+        <v/>
+      </c>
+      <c r="L26" s="22">
+        <f>IF(L21=$C$6,$C$9,IF(L21&gt;$C$6,L23*0.02,0))</f>
+        <v/>
+      </c>
+      <c r="M26" s="22">
+        <f>IF(M21=$C$6,$C$9,IF(M21&gt;$C$6,M23*0.02,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Equity Value (£)</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="22">
+        <f>IF(D21&lt;=$C$6,D24+D25+D26,C27*(1+$C$14))</f>
+        <v/>
+      </c>
+      <c r="E27" s="22">
+        <f>IF(E21&lt;=$C$6,E24+E25+E26,D27*(1+$C$14))</f>
+        <v/>
+      </c>
+      <c r="F27" s="22">
+        <f>IF(F21&lt;=$C$6,F24+F25+F26,E27*(1+$C$14))</f>
+        <v/>
+      </c>
+      <c r="G27" s="22">
+        <f>IF(G21&lt;=$C$6,G24+G25+G26,F27*(1+$C$14))</f>
+        <v/>
+      </c>
+      <c r="H27" s="22">
+        <f>IF(H21&lt;=$C$6,H24+H25+H26,G27*(1+$C$14))</f>
+        <v/>
+      </c>
+      <c r="I27" s="22">
+        <f>IF(I21&lt;=$C$6,I24+I25+I26,H27*(1+$C$14))</f>
+        <v/>
+      </c>
+      <c r="J27" s="22">
+        <f>IF(J21&lt;=$C$6,J24+J25+J26,I27*(1+$C$14))</f>
+        <v/>
+      </c>
+      <c r="K27" s="22">
+        <f>IF(K21&lt;=$C$6,K24+K25+K26,J27*(1+$C$14))</f>
+        <v/>
+      </c>
+      <c r="L27" s="22">
+        <f>IF(L21&lt;=$C$6,L24+L25+L26,K27*(1+$C$14))</f>
+        <v/>
+      </c>
+      <c r="M27" s="22">
+        <f>IF(M21&lt;=$C$6,M24+M25+M26,L27*(1+$C$14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Discount Rate (tiered)</t>
+        </is>
+      </c>
+      <c r="C28" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="36">
+        <f>IF(D21&lt;=3,$C$10,IF(D21&lt;=6,$C$11,$C$12))</f>
+        <v/>
+      </c>
+      <c r="E28" s="36">
+        <f>IF(E21&lt;=3,$C$10,IF(E21&lt;=6,$C$11,$C$12))</f>
+        <v/>
+      </c>
+      <c r="F28" s="36">
+        <f>IF(F21&lt;=3,$C$10,IF(F21&lt;=6,$C$11,$C$12))</f>
+        <v/>
+      </c>
+      <c r="G28" s="36">
+        <f>IF(G21&lt;=3,$C$10,IF(G21&lt;=6,$C$11,$C$12))</f>
+        <v/>
+      </c>
+      <c r="H28" s="36">
+        <f>IF(H21&lt;=3,$C$10,IF(H21&lt;=6,$C$11,$C$12))</f>
+        <v/>
+      </c>
+      <c r="I28" s="36">
+        <f>IF(I21&lt;=3,$C$10,IF(I21&lt;=6,$C$11,$C$12))</f>
+        <v/>
+      </c>
+      <c r="J28" s="36">
+        <f>IF(J21&lt;=3,$C$10,IF(J21&lt;=6,$C$11,$C$12))</f>
+        <v/>
+      </c>
+      <c r="K28" s="36">
+        <f>IF(K21&lt;=3,$C$10,IF(K21&lt;=6,$C$11,$C$12))</f>
+        <v/>
+      </c>
+      <c r="L28" s="36">
+        <f>IF(L21&lt;=3,$C$10,IF(L21&lt;=6,$C$11,$C$12))</f>
+        <v/>
+      </c>
+      <c r="M28" s="36">
+        <f>IF(M21&lt;=3,$C$10,IF(M21&lt;=6,$C$11,$C$12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Discount Period (years from valuation date)</t>
+        </is>
+      </c>
+      <c r="C29" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="37">
+        <f>C29+ROUND((D22-C22)/365,1)</f>
+        <v/>
+      </c>
+      <c r="E29" s="37">
+        <f>D29+ROUND((E22-D22)/365,1)</f>
+        <v/>
+      </c>
+      <c r="F29" s="37">
+        <f>E29+ROUND((F22-E22)/365,1)</f>
+        <v/>
+      </c>
+      <c r="G29" s="37">
+        <f>F29+ROUND((G22-F22)/365,1)</f>
+        <v/>
+      </c>
+      <c r="H29" s="37">
+        <f>G29+ROUND((H22-G22)/365,1)</f>
+        <v/>
+      </c>
+      <c r="I29" s="37">
+        <f>H29+ROUND((I22-H22)/365,1)</f>
+        <v/>
+      </c>
+      <c r="J29" s="37">
+        <f>I29+ROUND((J22-I22)/365,1)</f>
+        <v/>
+      </c>
+      <c r="K29" s="37">
+        <f>J29+ROUND((K22-J22)/365,1)</f>
+        <v/>
+      </c>
+      <c r="L29" s="37">
+        <f>K29+ROUND((L22-K22)/365,1)</f>
+        <v/>
+      </c>
+      <c r="M29" s="37">
+        <f>L29+ROUND((M22-L22)/365,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Discount Factor</t>
+        </is>
+      </c>
+      <c r="C30" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="38">
+        <f>1/(1+D28)^D29</f>
+        <v/>
+      </c>
+      <c r="E30" s="38">
+        <f>1/(1+E28)^E29</f>
+        <v/>
+      </c>
+      <c r="F30" s="38">
+        <f>1/(1+F28)^F29</f>
+        <v/>
+      </c>
+      <c r="G30" s="38">
+        <f>1/(1+G28)^G29</f>
+        <v/>
+      </c>
+      <c r="H30" s="38">
+        <f>1/(1+H28)^H29</f>
+        <v/>
+      </c>
+      <c r="I30" s="38">
+        <f>1/(1+I28)^I29</f>
+        <v/>
+      </c>
+      <c r="J30" s="38">
+        <f>1/(1+J28)^J29</f>
+        <v/>
+      </c>
+      <c r="K30" s="38">
+        <f>1/(1+K28)^K29</f>
+        <v/>
+      </c>
+      <c r="L30" s="38">
+        <f>1/(1+L28)^L29</f>
+        <v/>
+      </c>
+      <c r="M30" s="38">
+        <f>1/(1+M28)^M29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Present Value (£) — exit year onwards</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="inlineStr"/>
+      <c r="D31" s="22" t="inlineStr"/>
+      <c r="E31" s="22" t="inlineStr"/>
+      <c r="F31" s="22" t="inlineStr"/>
+      <c r="G31" s="22" t="inlineStr"/>
+      <c r="H31" s="22">
+        <f>H27/((1+$C$10)^MIN(5,3)*(1+$C$11)^MAX(0,MIN(5,6)-3)*(1+$C$12)^MAX(0,5-6))</f>
+        <v/>
+      </c>
+      <c r="I31" s="22">
+        <f>I27/((1+$C$10)^MIN(6,3)*(1+$C$11)^MAX(0,MIN(6,6)-3)*(1+$C$12)^MAX(0,6-6))</f>
+        <v/>
+      </c>
+      <c r="J31" s="22">
+        <f>J27/((1+$C$10)^MIN(7,3)*(1+$C$11)^MAX(0,MIN(7,6)-3)*(1+$C$12)^MAX(0,7-6))</f>
+        <v/>
+      </c>
+      <c r="K31" s="22">
+        <f>K27/((1+$C$10)^MIN(8,3)*(1+$C$11)^MAX(0,MIN(8,6)-3)*(1+$C$12)^MAX(0,8-6))</f>
+        <v/>
+      </c>
+      <c r="L31" s="22">
+        <f>L27/((1+$C$10)^MIN(9,3)*(1+$C$11)^MAX(0,MIN(9,6)-3)*(1+$C$12)^MAX(0,9-6))</f>
+        <v/>
+      </c>
+      <c r="M31" s="22">
+        <f>M27/((1+$C$10)^MIN(10,3)*(1+$C$11)^MAX(0,MIN(10,6)-3)*(1+$C$12)^MAX(0,10-6))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>D. INVESTOR CALCULATION</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="n"/>
+      <c r="K33" s="2" t="n"/>
+      <c r="L33" s="2" t="n"/>
+      <c r="M33" s="2" t="n"/>
+      <c r="N33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Investment Amount (£)</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="n">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Equity Stake at Entry</t>
+        </is>
+      </c>
+      <c r="C35" s="39">
+        <f>'Cap Table'!C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Dilution Effect</t>
+        </is>
+      </c>
+      <c r="C36" s="39">
+        <f>'Cap Table'!C30-'Cap Table'!C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Equity Stake at Exit</t>
+        </is>
+      </c>
+      <c r="C37" s="40">
+        <f>$C$35+$C$36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Exit Proceeds  (Equity Value × Stake at Exit)</t>
+        </is>
+      </c>
+      <c r="C38" s="22">
+        <f>H27*$C$37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Investor Cash Flows (£)</t>
+        </is>
+      </c>
+      <c r="C39" s="22">
+        <f>-$C$34</f>
+        <v/>
+      </c>
+      <c r="D39" s="22">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="E39" s="22">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="F39" s="22">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="G39" s="22">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="H39" s="22">
+        <f>$C$38</f>
+        <v/>
+      </c>
+      <c r="I39" s="22">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="J39" s="22">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="K39" s="22">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="L39" s="22">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="M39" s="22">
+        <f>0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Investor IRR  (=IRR of cash flows)</t>
+        </is>
+      </c>
+      <c r="C40" s="40">
+        <f>IRR(C39:M39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Cash-on-Cash Multiple  (Exit Proceeds ÷ Investment)</t>
+        </is>
+      </c>
+      <c r="C41" s="41">
+        <f>$C$38/$C$34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>E. SUMMARY METRICS</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
+      <c r="I43" s="2" t="n"/>
+      <c r="J43" s="2" t="n"/>
+      <c r="K43" s="2" t="n"/>
+      <c r="L43" s="2" t="n"/>
+      <c r="M43" s="2" t="n"/>
+      <c r="N43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Equity Value Today (£)</t>
+        </is>
+      </c>
+      <c r="C44" s="42">
+        <f>H31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Investor IRR</t>
+        </is>
+      </c>
+      <c r="C45" s="43">
+        <f>$C$40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Cash-on-Cash Multiple</t>
+        </is>
+      </c>
+      <c r="C46" s="44">
+        <f>$C$41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Exit Proceeds (Year 5, £)</t>
+        </is>
+      </c>
+      <c r="C47" s="42">
+        <f>$C$38</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="007030A0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:K36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>CAPITALISATION TABLE  (CAP TABLE)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Share counts are fractional — rounded for display only</t>
+        </is>
+      </c>
+      <c r="I2" s="45" t="inlineStr">
+        <is>
+          <t>GBP/USD FX Rate:</t>
+        </is>
+      </c>
+      <c r="J2" s="46" t="n">
+        <v>0.7577</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>A. INITIAL CAP TABLE  (Pre-Funding)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Shareholder</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Shares</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Ownership %</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="47" t="inlineStr">
+        <is>
+          <t>Founders</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="C5" s="40">
+        <f>B5/B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>B. FUNDING ROUNDS</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Ownership %</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Shares Issued</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Amount (£)</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Amount ($)</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Valuation (£)</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Valuation ($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="47" t="inlineStr">
+        <is>
+          <t>Pre-seed T1</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="C9" s="49" t="n">
+        <v>0.040652</v>
+      </c>
+      <c r="D9" s="50">
+        <f>(B5)/(1-C9)-(B5)</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>Assumptions!C52</f>
+        <v/>
+      </c>
+      <c r="F9" s="22">
+        <f>E9/$J$2</f>
+        <v/>
+      </c>
+      <c r="G9" s="22">
+        <f>E9/C9</f>
+        <v/>
+      </c>
+      <c r="H9" s="22">
+        <f>G9/$J$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="47" t="inlineStr">
+        <is>
+          <t>Pre-seed T2</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="C10" s="49" t="n">
+        <v>0.029269</v>
+      </c>
+      <c r="D10" s="50">
+        <f>(B5+SUM(D9:D9))/(1-C10)-(B5+SUM(D9:D9))</f>
+        <v/>
+      </c>
+      <c r="E10" s="19">
+        <f>Assumptions!D52</f>
+        <v/>
+      </c>
+      <c r="F10" s="22">
+        <f>E10/$J$2</f>
+        <v/>
+      </c>
+      <c r="G10" s="22">
+        <f>E10/C10</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>G10/$J$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="47" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C11" s="49" t="n">
+        <v>0.1372</v>
+      </c>
+      <c r="D11" s="50">
+        <f>(B5+SUM(D9:D10))/(1-C11)-(B5+SUM(D9:D10))</f>
+        <v/>
+      </c>
+      <c r="E11" s="19">
+        <f>Assumptions!D52</f>
+        <v/>
+      </c>
+      <c r="F11" s="22">
+        <f>E11/$J$2</f>
+        <v/>
+      </c>
+      <c r="G11" s="22">
+        <f>E11/C11</f>
+        <v/>
+      </c>
+      <c r="H11" s="22">
+        <f>G11/$J$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="47" t="inlineStr">
+        <is>
+          <t>Series A T1</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>2027-10-01</t>
+        </is>
+      </c>
+      <c r="C12" s="49" t="n">
+        <v>0.095278</v>
+      </c>
+      <c r="D12" s="50">
+        <f>(B5+SUM(D9:D11))/(1-C12)-(B5+SUM(D9:D11))</f>
+        <v/>
+      </c>
+      <c r="E12" s="19">
+        <f>Assumptions!E52</f>
+        <v/>
+      </c>
+      <c r="F12" s="22">
+        <f>E12/$J$2</f>
+        <v/>
+      </c>
+      <c r="G12" s="22">
+        <f>E12/C12</f>
+        <v/>
+      </c>
+      <c r="H12" s="22">
+        <f>G12/$J$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="47" t="inlineStr">
+        <is>
+          <t>Series A T2</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>2028-10-01</t>
+        </is>
+      </c>
+      <c r="C13" s="49" t="n">
+        <v>0.049624</v>
+      </c>
+      <c r="D13" s="50">
+        <f>(B5+SUM(D9:D12))/(1-C13)-(B5+SUM(D9:D12))</f>
+        <v/>
+      </c>
+      <c r="E13" s="19">
+        <f>Assumptions!F52</f>
+        <v/>
+      </c>
+      <c r="F13" s="22">
+        <f>E13/$J$2</f>
+        <v/>
+      </c>
+      <c r="G13" s="22">
+        <f>E13/C13</f>
+        <v/>
+      </c>
+      <c r="H13" s="22">
+        <f>G13/$J$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="47" t="inlineStr">
+        <is>
+          <t>Series B</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>2029-10-01</t>
+        </is>
+      </c>
+      <c r="C14" s="49" t="n">
+        <v>0.129228</v>
+      </c>
+      <c r="D14" s="50">
+        <f>(B5+SUM(D9:D13))/(1-C14)-(B5+SUM(D9:D13))</f>
+        <v/>
+      </c>
+      <c r="E14" s="19">
+        <f>Assumptions!G52</f>
+        <v/>
+      </c>
+      <c r="F14" s="22">
+        <f>E14/$J$2</f>
+        <v/>
+      </c>
+      <c r="G14" s="22">
+        <f>E14/C14</f>
+        <v/>
+      </c>
+      <c r="H14" s="22">
+        <f>G14/$J$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>C. CUMULATIVE CAP TABLE  (Shares after each round)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Shareholder</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Founders</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Pre-seed T1</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Pre-seed T2</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Series A T1</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>Series A T2</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Series B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Founders</t>
+        </is>
+      </c>
+      <c r="B18" s="50">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="C18" s="50">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="D18" s="50">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="E18" s="50">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="F18" s="50">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="G18" s="50">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="H18" s="50">
+        <f>$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Pre-seed T1</t>
+        </is>
+      </c>
+      <c r="B19" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="50">
+        <f>$D$9</f>
+        <v/>
+      </c>
+      <c r="D19" s="50">
+        <f>$D$9</f>
+        <v/>
+      </c>
+      <c r="E19" s="50">
+        <f>$D$9</f>
+        <v/>
+      </c>
+      <c r="F19" s="50">
+        <f>$D$9</f>
+        <v/>
+      </c>
+      <c r="G19" s="50">
+        <f>$D$9</f>
+        <v/>
+      </c>
+      <c r="H19" s="50">
+        <f>$D$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Pre-seed T2</t>
+        </is>
+      </c>
+      <c r="B20" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="50">
+        <f>$D$10</f>
+        <v/>
+      </c>
+      <c r="E20" s="50">
+        <f>$D$10</f>
+        <v/>
+      </c>
+      <c r="F20" s="50">
+        <f>$D$10</f>
+        <v/>
+      </c>
+      <c r="G20" s="50">
+        <f>$D$10</f>
+        <v/>
+      </c>
+      <c r="H20" s="50">
+        <f>$D$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B21" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="50">
+        <f>$D$11</f>
+        <v/>
+      </c>
+      <c r="F21" s="50">
+        <f>$D$11</f>
+        <v/>
+      </c>
+      <c r="G21" s="50">
+        <f>$D$11</f>
+        <v/>
+      </c>
+      <c r="H21" s="50">
+        <f>$D$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Series A T1</t>
+        </is>
+      </c>
+      <c r="B22" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="50">
+        <f>$D$12</f>
+        <v/>
+      </c>
+      <c r="G22" s="50">
+        <f>$D$12</f>
+        <v/>
+      </c>
+      <c r="H22" s="50">
+        <f>$D$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Series A T2</t>
+        </is>
+      </c>
+      <c r="B23" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="50">
+        <f>$D$13</f>
+        <v/>
+      </c>
+      <c r="H23" s="50">
+        <f>$D$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Series B</t>
+        </is>
+      </c>
+      <c r="B24" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="50">
+        <f>$D$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>TOTAL SHARES</t>
+        </is>
+      </c>
+      <c r="B25" s="51">
+        <f>SUM(B18:B24)</f>
+        <v/>
+      </c>
+      <c r="C25" s="51">
+        <f>SUM(C18:C24)</f>
+        <v/>
+      </c>
+      <c r="D25" s="51">
+        <f>SUM(D18:D24)</f>
+        <v/>
+      </c>
+      <c r="E25" s="51">
+        <f>SUM(E18:E24)</f>
+        <v/>
+      </c>
+      <c r="F25" s="51">
+        <f>SUM(F18:F24)</f>
+        <v/>
+      </c>
+      <c r="G25" s="51">
+        <f>SUM(G18:G24)</f>
+        <v/>
+      </c>
+      <c r="H25" s="51">
+        <f>SUM(H18:H24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>D. FINAL OWNERSHIP %  (After All Rounds)</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="2" t="n"/>
+      <c r="J27" s="2" t="n"/>
+      <c r="K27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Shareholder</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Shares Held</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Ownership %</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Founders</t>
+        </is>
+      </c>
+      <c r="B29" s="50">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="C29" s="40">
+        <f>B29/H25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Pre-seed T1</t>
+        </is>
+      </c>
+      <c r="B30" s="50">
+        <f>$D$9</f>
+        <v/>
+      </c>
+      <c r="C30" s="40">
+        <f>B30/H25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Pre-seed T2</t>
+        </is>
+      </c>
+      <c r="B31" s="50">
+        <f>$D$10</f>
+        <v/>
+      </c>
+      <c r="C31" s="40">
+        <f>B31/H25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B32" s="50">
+        <f>$D$11</f>
+        <v/>
+      </c>
+      <c r="C32" s="40">
+        <f>B32/H25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Series A T1</t>
+        </is>
+      </c>
+      <c r="B33" s="50">
+        <f>$D$12</f>
+        <v/>
+      </c>
+      <c r="C33" s="40">
+        <f>B33/H25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Series A T2</t>
+        </is>
+      </c>
+      <c r="B34" s="50">
+        <f>$D$13</f>
+        <v/>
+      </c>
+      <c r="C34" s="40">
+        <f>B34/H25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Series B</t>
+        </is>
+      </c>
+      <c r="B35" s="50">
+        <f>$D$14</f>
+        <v/>
+      </c>
+      <c r="C35" s="40">
+        <f>B35/H25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="23" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B36" s="51">
+        <f>H25</f>
+        <v/>
+      </c>
+      <c r="C36" s="52">
+        <f>SUM(C29:C35)</f>
+        <v/>
+      </c>
+      <c r="D36" s="24" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Cap Table valuation links and add Investor Dashboard sheet
Agent-Logs-Url: https://github.com/DejAmour/Joule-Financial-Model/sessions/a4871153-9b83-4e89-95ff-fcaea5c2ac53

Co-authored-by: DejAmour <159169578+DejAmour@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/financial_model.xlsx
+++ b/financial_model.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Cash Flow" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Valuation" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Cap Table" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Dashboard" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Assumptions'!$1:$3</definedName>
@@ -23,6 +24,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Cash Flow'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Valuation'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Cap Table'!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Dashboard'!$1:$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -30,7 +32,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="£#,##0.00"/>
     <numFmt numFmtId="166" formatCode="£#,##0"/>
@@ -40,8 +42,9 @@
     <numFmt numFmtId="170" formatCode="0.0000"/>
     <numFmt numFmtId="171" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="172" formatCode="0.0000%"/>
+    <numFmt numFmtId="173" formatCode="0&quot; years&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,8 +98,43 @@
       <color rgb="001F4E79"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -121,6 +159,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000B050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -163,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -307,6 +355,59 @@
     <xf numFmtId="164" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -381,6 +482,808 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Scenario Comparison: Total Gross Revenue</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!B5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="20000">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$6:$A$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$B$6:$B$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!C5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="20000">
+              <a:solidFill>
+                <a:srgbClr val="1F4E79"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$6:$A$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$C$6:$C$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!D5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="20000">
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$6:$A$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$D$6:$D$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Revenue (£)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Revenue Streams Breakdown</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <areaChart>
+        <grouping val="stacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!O5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F4E79"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$N$6:$N$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$O$6:$O$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!P5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E75B6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$N$6:$N$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$P$6:$P$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!Q5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="00B050"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$N$6:$N$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$Q$6:$Q$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </areaChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Revenue (£)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>kWh Revenue: 15-Year Projection (2026–2040)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!B22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="20000">
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$23:$A$37</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$B$23:$B$37</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>kWh Revenue (£)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Core Financials: EBIT &amp; Net Income</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!O22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1F4E79"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$N$23:$N$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$O$23:$O$27</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!P22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="00B050"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$N$23:$N$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$P$23:$P$27</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Profit (£)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Targeted Funds Raised (Base Case)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!B39</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E75B6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$40:$A$44</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$B$40:$B$44</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Funds Raised (£)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cap Table: Final Ownership Distribution</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!B56</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$57:$A$63</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$B$57:$B$63</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
 </file>
 
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -669,6 +1572,42 @@
   This ensures investors receive exactly their target post-round ownership %.</t>
       </text>
     </comment>
+    <comment ref="G9" authorId="0" shapeId="0">
+      <text>
+        <t>Linked to Valuation sheet Enterprise Value (row 24, col C).
+EV = Revenue × 7x multiple.</t>
+      </text>
+    </comment>
+    <comment ref="G10" authorId="0" shapeId="0">
+      <text>
+        <t>Linked to Valuation sheet Enterprise Value (row 24, col D).
+EV = Revenue × 7x multiple.</t>
+      </text>
+    </comment>
+    <comment ref="G11" authorId="0" shapeId="0">
+      <text>
+        <t>Linked to Valuation sheet Enterprise Value (row 24, col D).
+EV = Revenue × 7x multiple.</t>
+      </text>
+    </comment>
+    <comment ref="G12" authorId="0" shapeId="0">
+      <text>
+        <t>Linked to Valuation sheet Enterprise Value (row 24, col E).
+EV = Revenue × 7x multiple.</t>
+      </text>
+    </comment>
+    <comment ref="G13" authorId="0" shapeId="0">
+      <text>
+        <t>Linked to Valuation sheet Enterprise Value (row 24, col F).
+EV = Revenue × 7x multiple.</t>
+      </text>
+    </comment>
+    <comment ref="G14" authorId="0" shapeId="0">
+      <text>
+        <t>Linked to Valuation sheet Enterprise Value (row 24, col G).
+EV = Revenue × 7x multiple.</t>
+      </text>
+    </comment>
     <comment ref="C36" authorId="0" shapeId="0">
       <text>
         <t>Should equal 100%. If not, check shares-issued formulas.</t>
@@ -676,6 +1615,143 @@
     </comment>
   </commentList>
 </comments>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>17</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>17</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>55</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4928,8 +6004,8 @@
         <f>E9/$J$2</f>
         <v/>
       </c>
-      <c r="G9" s="22">
-        <f>E9/C9</f>
+      <c r="G9" s="19">
+        <f>Valuation!C24</f>
         <v/>
       </c>
       <c r="H9" s="22">
@@ -4963,8 +6039,8 @@
         <f>E10/$J$2</f>
         <v/>
       </c>
-      <c r="G10" s="22">
-        <f>E10/C10</f>
+      <c r="G10" s="19">
+        <f>Valuation!D24</f>
         <v/>
       </c>
       <c r="H10" s="22">
@@ -4998,8 +6074,8 @@
         <f>E11/$J$2</f>
         <v/>
       </c>
-      <c r="G11" s="22">
-        <f>E11/C11</f>
+      <c r="G11" s="19">
+        <f>Valuation!D24</f>
         <v/>
       </c>
       <c r="H11" s="22">
@@ -5033,8 +6109,8 @@
         <f>E12/$J$2</f>
         <v/>
       </c>
-      <c r="G12" s="22">
-        <f>E12/C12</f>
+      <c r="G12" s="19">
+        <f>Valuation!E24</f>
         <v/>
       </c>
       <c r="H12" s="22">
@@ -5068,8 +6144,8 @@
         <f>E13/$J$2</f>
         <v/>
       </c>
-      <c r="G13" s="22">
-        <f>E13/C13</f>
+      <c r="G13" s="19">
+        <f>Valuation!F24</f>
         <v/>
       </c>
       <c r="H13" s="22">
@@ -5103,8 +6179,8 @@
         <f>E14/$J$2</f>
         <v/>
       </c>
-      <c r="G14" s="22">
-        <f>E14/C14</f>
+      <c r="G14" s="19">
+        <f>Valuation!G24</f>
         <v/>
       </c>
       <c r="H14" s="22">
@@ -5590,4 +6666,1177 @@
   <pageSetup orientation="landscape" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0000B050"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:S95"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="53" t="inlineStr">
+        <is>
+          <t>JOULE FINANCIAL MODEL — INVESTOR DASHBOARD</t>
+        </is>
+      </c>
+      <c r="B1" s="54" t="n"/>
+      <c r="C1" s="54" t="n"/>
+      <c r="D1" s="54" t="n"/>
+      <c r="E1" s="54" t="n"/>
+      <c r="F1" s="54" t="n"/>
+      <c r="G1" s="54" t="n"/>
+      <c r="H1" s="54" t="n"/>
+      <c r="I1" s="54" t="n"/>
+      <c r="J1" s="54" t="n"/>
+      <c r="K1" s="54" t="n"/>
+      <c r="L1" s="54" t="n"/>
+      <c r="M1" s="54" t="n"/>
+      <c r="N1" s="54" t="n"/>
+      <c r="O1" s="54" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="55" t="inlineStr">
+        <is>
+          <t>Equity Value Today (£)</t>
+        </is>
+      </c>
+      <c r="B2" s="56">
+        <f>IF(ISNUMBER(Valuation!C44),Valuation!C44,"N/A")</f>
+        <v/>
+      </c>
+      <c r="D2" s="55" t="inlineStr">
+        <is>
+          <t>Exit Valuation Year 5 (£)</t>
+        </is>
+      </c>
+      <c r="E2" s="56">
+        <f>IF(ISNUMBER(Valuation!H27),Valuation!H27,"N/A")</f>
+        <v/>
+      </c>
+      <c r="G2" s="55" t="inlineStr">
+        <is>
+          <t>Investor IRR</t>
+        </is>
+      </c>
+      <c r="H2" s="57">
+        <f>IF(ISNUMBER(Valuation!C45),Valuation!C45,"N/A")</f>
+        <v/>
+      </c>
+      <c r="J2" s="55" t="inlineStr">
+        <is>
+          <t>Cash-on-Cash Multiple</t>
+        </is>
+      </c>
+      <c r="K2" s="58">
+        <f>IF(ISNUMBER(Valuation!C46),Valuation!C46,"N/A")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="55" t="inlineStr">
+        <is>
+          <t>EV/Revenue Multiple</t>
+        </is>
+      </c>
+      <c r="B3" s="59" t="n">
+        <v>7</v>
+      </c>
+      <c r="D3" s="55" t="inlineStr">
+        <is>
+          <t>Model Exit Year</t>
+        </is>
+      </c>
+      <c r="E3" s="60" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" s="55" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="H3" s="61">
+        <f>Assumptions!C4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Worst</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Best</t>
+        </is>
+      </c>
+      <c r="N5" s="9" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>Upfront Fee</t>
+        </is>
+      </c>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>Completion</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>kWh Revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B6" s="19">
+        <f>Scenarios!C9</f>
+        <v/>
+      </c>
+      <c r="C6" s="19">
+        <f>Scenarios!C13</f>
+        <v/>
+      </c>
+      <c r="D6" s="19">
+        <f>Scenarios!C17</f>
+        <v/>
+      </c>
+      <c r="N6" s="20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="O6" s="19">
+        <f>'Income Statement'!C7</f>
+        <v/>
+      </c>
+      <c r="P6" s="19">
+        <f>'Income Statement'!C8</f>
+        <v/>
+      </c>
+      <c r="Q6" s="19">
+        <f>'Income Statement'!C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B7" s="19">
+        <f>Scenarios!D9</f>
+        <v/>
+      </c>
+      <c r="C7" s="19">
+        <f>Scenarios!D13</f>
+        <v/>
+      </c>
+      <c r="D7" s="19">
+        <f>Scenarios!D17</f>
+        <v/>
+      </c>
+      <c r="N7" s="20" t="n">
+        <v>2027</v>
+      </c>
+      <c r="O7" s="19">
+        <f>'Income Statement'!D7</f>
+        <v/>
+      </c>
+      <c r="P7" s="19">
+        <f>'Income Statement'!D8</f>
+        <v/>
+      </c>
+      <c r="Q7" s="19">
+        <f>'Income Statement'!D9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B8" s="19">
+        <f>Scenarios!E9</f>
+        <v/>
+      </c>
+      <c r="C8" s="19">
+        <f>Scenarios!E13</f>
+        <v/>
+      </c>
+      <c r="D8" s="19">
+        <f>Scenarios!E17</f>
+        <v/>
+      </c>
+      <c r="N8" s="20" t="n">
+        <v>2028</v>
+      </c>
+      <c r="O8" s="19">
+        <f>'Income Statement'!E7</f>
+        <v/>
+      </c>
+      <c r="P8" s="19">
+        <f>'Income Statement'!E8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="19">
+        <f>'Income Statement'!E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="n">
+        <v>2029</v>
+      </c>
+      <c r="B9" s="19">
+        <f>Scenarios!F9</f>
+        <v/>
+      </c>
+      <c r="C9" s="19">
+        <f>Scenarios!F13</f>
+        <v/>
+      </c>
+      <c r="D9" s="19">
+        <f>Scenarios!F17</f>
+        <v/>
+      </c>
+      <c r="N9" s="20" t="n">
+        <v>2029</v>
+      </c>
+      <c r="O9" s="19">
+        <f>'Income Statement'!F7</f>
+        <v/>
+      </c>
+      <c r="P9" s="19">
+        <f>'Income Statement'!F8</f>
+        <v/>
+      </c>
+      <c r="Q9" s="19">
+        <f>'Income Statement'!F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="n">
+        <v>2030</v>
+      </c>
+      <c r="B10" s="19">
+        <f>Scenarios!G9</f>
+        <v/>
+      </c>
+      <c r="C10" s="19">
+        <f>Scenarios!G13</f>
+        <v/>
+      </c>
+      <c r="D10" s="19">
+        <f>Scenarios!G17</f>
+        <v/>
+      </c>
+      <c r="N10" s="20" t="n">
+        <v>2030</v>
+      </c>
+      <c r="O10" s="19">
+        <f>'Income Statement'!G7</f>
+        <v/>
+      </c>
+      <c r="P10" s="19">
+        <f>'Income Statement'!G8</f>
+        <v/>
+      </c>
+      <c r="Q10" s="19">
+        <f>'Income Statement'!G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Year (15yr)</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>kWh Revenue</t>
+        </is>
+      </c>
+      <c r="N22" s="9" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="O22" s="9" t="inlineStr">
+        <is>
+          <t>EBIT</t>
+        </is>
+      </c>
+      <c r="P22" s="9" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="20">
+        <f>A81</f>
+        <v/>
+      </c>
+      <c r="B23" s="22">
+        <f>C81</f>
+        <v/>
+      </c>
+      <c r="N23" s="20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="O23" s="19">
+        <f>'Income Statement'!C27</f>
+        <v/>
+      </c>
+      <c r="P23" s="19">
+        <f>'Income Statement'!C36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="20">
+        <f>A82</f>
+        <v/>
+      </c>
+      <c r="B24" s="22">
+        <f>C82</f>
+        <v/>
+      </c>
+      <c r="N24" s="20" t="n">
+        <v>2027</v>
+      </c>
+      <c r="O24" s="19">
+        <f>'Income Statement'!D27</f>
+        <v/>
+      </c>
+      <c r="P24" s="19">
+        <f>'Income Statement'!D36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20">
+        <f>A83</f>
+        <v/>
+      </c>
+      <c r="B25" s="22">
+        <f>C83</f>
+        <v/>
+      </c>
+      <c r="N25" s="20" t="n">
+        <v>2028</v>
+      </c>
+      <c r="O25" s="19">
+        <f>'Income Statement'!E27</f>
+        <v/>
+      </c>
+      <c r="P25" s="19">
+        <f>'Income Statement'!E36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20">
+        <f>A84</f>
+        <v/>
+      </c>
+      <c r="B26" s="22">
+        <f>C84</f>
+        <v/>
+      </c>
+      <c r="N26" s="20" t="n">
+        <v>2029</v>
+      </c>
+      <c r="O26" s="19">
+        <f>'Income Statement'!F27</f>
+        <v/>
+      </c>
+      <c r="P26" s="19">
+        <f>'Income Statement'!F36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="20">
+        <f>A85</f>
+        <v/>
+      </c>
+      <c r="B27" s="22">
+        <f>C85</f>
+        <v/>
+      </c>
+      <c r="N27" s="20" t="n">
+        <v>2030</v>
+      </c>
+      <c r="O27" s="19">
+        <f>'Income Statement'!G27</f>
+        <v/>
+      </c>
+      <c r="P27" s="19">
+        <f>'Income Statement'!G36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="20">
+        <f>A86</f>
+        <v/>
+      </c>
+      <c r="B28" s="22">
+        <f>C86</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="20">
+        <f>A87</f>
+        <v/>
+      </c>
+      <c r="B29" s="22">
+        <f>C87</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="20">
+        <f>A88</f>
+        <v/>
+      </c>
+      <c r="B30" s="22">
+        <f>C88</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="20">
+        <f>A89</f>
+        <v/>
+      </c>
+      <c r="B31" s="22">
+        <f>C89</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="20">
+        <f>A90</f>
+        <v/>
+      </c>
+      <c r="B32" s="22">
+        <f>C90</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="20">
+        <f>A91</f>
+        <v/>
+      </c>
+      <c r="B33" s="22">
+        <f>C91</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="20">
+        <f>A92</f>
+        <v/>
+      </c>
+      <c r="B34" s="22">
+        <f>C92</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="20">
+        <f>A93</f>
+        <v/>
+      </c>
+      <c r="B35" s="22">
+        <f>C93</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="20">
+        <f>A94</f>
+        <v/>
+      </c>
+      <c r="B36" s="22">
+        <f>C94</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="20">
+        <f>A95</f>
+        <v/>
+      </c>
+      <c r="B37" s="22">
+        <f>C95</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Funds Raised</t>
+        </is>
+      </c>
+      <c r="N39" s="62" t="inlineStr">
+        <is>
+          <t>KEY VALUATION METRICS</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="n"/>
+      <c r="P39" s="2" t="n"/>
+      <c r="Q39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B40" s="19">
+        <f>Scenarios!C12</f>
+        <v/>
+      </c>
+      <c r="N40" s="8" t="inlineStr">
+        <is>
+          <t>Equity Value Today</t>
+        </is>
+      </c>
+      <c r="O40" s="63">
+        <f>IF(ISNUMBER(Valuation!C44),Valuation!C44,0)</f>
+        <v/>
+      </c>
+      <c r="P40" s="64" t="n"/>
+      <c r="Q40" s="64" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="20" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B41" s="19">
+        <f>Scenarios!D12</f>
+        <v/>
+      </c>
+      <c r="N41" s="8" t="inlineStr">
+        <is>
+          <t>Exit Valuation (Year 5)</t>
+        </is>
+      </c>
+      <c r="O41" s="63">
+        <f>IF(ISNUMBER(Valuation!H27),Valuation!H27,0)</f>
+        <v/>
+      </c>
+      <c r="P41" s="64" t="n"/>
+      <c r="Q41" s="64" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B42" s="19">
+        <f>Scenarios!E12</f>
+        <v/>
+      </c>
+      <c r="N42" s="8" t="inlineStr">
+        <is>
+          <t>Investor IRR</t>
+        </is>
+      </c>
+      <c r="O42" s="65">
+        <f>IF(ISNUMBER(Valuation!C45),Valuation!C45,0)</f>
+        <v/>
+      </c>
+      <c r="P42" s="64" t="n"/>
+      <c r="Q42" s="64" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="20" t="n">
+        <v>2029</v>
+      </c>
+      <c r="B43" s="19">
+        <f>Scenarios!F12</f>
+        <v/>
+      </c>
+      <c r="N43" s="8" t="inlineStr">
+        <is>
+          <t>Cash-on-Cash Multiple</t>
+        </is>
+      </c>
+      <c r="O43" s="66">
+        <f>IF(ISNUMBER(Valuation!C46),Valuation!C46,0)</f>
+        <v/>
+      </c>
+      <c r="P43" s="64" t="n"/>
+      <c r="Q43" s="64" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="20" t="n">
+        <v>2030</v>
+      </c>
+      <c r="B44" s="19">
+        <f>Scenarios!G12</f>
+        <v/>
+      </c>
+      <c r="N44" s="8" t="inlineStr">
+        <is>
+          <t>Exit Proceeds (£250K inv)</t>
+        </is>
+      </c>
+      <c r="O44" s="63">
+        <f>IF(ISNUMBER(Valuation!C47),Valuation!C47,0)</f>
+        <v/>
+      </c>
+      <c r="P44" s="64" t="n"/>
+      <c r="Q44" s="64" t="n"/>
+    </row>
+    <row r="45">
+      <c r="N45" s="8" t="inlineStr">
+        <is>
+          <t>EV/Revenue Multiple</t>
+        </is>
+      </c>
+      <c r="O45" s="67" t="n">
+        <v>7</v>
+      </c>
+      <c r="P45" s="64" t="n"/>
+      <c r="Q45" s="64" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>Shareholder</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>Ownership %</t>
+        </is>
+      </c>
+      <c r="N56" s="68" t="inlineStr">
+        <is>
+          <t>INVESTOR POTENTIAL RETURNS</t>
+        </is>
+      </c>
+      <c r="O56" s="54" t="n"/>
+      <c r="P56" s="54" t="n"/>
+      <c r="Q56" s="54" t="n"/>
+      <c r="R56" s="54" t="n"/>
+      <c r="S56" s="54" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Founders</t>
+        </is>
+      </c>
+      <c r="B57" s="39">
+        <f>'Cap Table'!C29</f>
+        <v/>
+      </c>
+      <c r="N57" s="69" t="inlineStr">
+        <is>
+          <t>Investment (£)</t>
+        </is>
+      </c>
+      <c r="O57" s="69" t="inlineStr">
+        <is>
+          <t>Equity at Entry</t>
+        </is>
+      </c>
+      <c r="P57" s="69" t="inlineStr">
+        <is>
+          <t>Equity at Exit</t>
+        </is>
+      </c>
+      <c r="Q57" s="69" t="inlineStr">
+        <is>
+          <t>Exit Proceeds (£)</t>
+        </is>
+      </c>
+      <c r="R57" s="69" t="inlineStr">
+        <is>
+          <t>Cash-on-Cash</t>
+        </is>
+      </c>
+      <c r="S57" s="69" t="inlineStr">
+        <is>
+          <t>IRR (Approx)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Pre-seed T1</t>
+        </is>
+      </c>
+      <c r="B58" s="39">
+        <f>'Cap Table'!C30</f>
+        <v/>
+      </c>
+      <c r="N58" s="10" t="n">
+        <v>50000</v>
+      </c>
+      <c r="O58" s="39">
+        <f>IF(Valuation!$C$34&gt;0,Valuation!$C$35*(N58/Valuation!$C$34),0)</f>
+        <v/>
+      </c>
+      <c r="P58" s="40">
+        <f>IF(AND(ISNUMBER(Valuation!$C$35),Valuation!$C$35&gt;0),O58*(Valuation!$C$37/Valuation!$C$35),0)</f>
+        <v/>
+      </c>
+      <c r="Q58" s="22">
+        <f>IF(ISNUMBER(Valuation!$H$27),P58*Valuation!$H$27,0)</f>
+        <v/>
+      </c>
+      <c r="R58" s="70">
+        <f>IF(N58&gt;0,Q58/N58,0)</f>
+        <v/>
+      </c>
+      <c r="S58" s="40">
+        <f>IF(Q58&gt;0,IRR({-N58,0,0,0,0,Q58}),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Pre-seed T2</t>
+        </is>
+      </c>
+      <c r="B59" s="39">
+        <f>'Cap Table'!C31</f>
+        <v/>
+      </c>
+      <c r="N59" s="10" t="n">
+        <v>100000</v>
+      </c>
+      <c r="O59" s="39">
+        <f>IF(Valuation!$C$34&gt;0,Valuation!$C$35*(N59/Valuation!$C$34),0)</f>
+        <v/>
+      </c>
+      <c r="P59" s="40">
+        <f>IF(AND(ISNUMBER(Valuation!$C$35),Valuation!$C$35&gt;0),O59*(Valuation!$C$37/Valuation!$C$35),0)</f>
+        <v/>
+      </c>
+      <c r="Q59" s="22">
+        <f>IF(ISNUMBER(Valuation!$H$27),P59*Valuation!$H$27,0)</f>
+        <v/>
+      </c>
+      <c r="R59" s="70">
+        <f>IF(N59&gt;0,Q59/N59,0)</f>
+        <v/>
+      </c>
+      <c r="S59" s="40">
+        <f>IF(Q59&gt;0,IRR({-N59,0,0,0,0,Q59}),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="B60" s="39">
+        <f>'Cap Table'!C32</f>
+        <v/>
+      </c>
+      <c r="N60" s="10" t="n">
+        <v>250000</v>
+      </c>
+      <c r="O60" s="39">
+        <f>IF(Valuation!$C$34&gt;0,Valuation!$C$35*(N60/Valuation!$C$34),0)</f>
+        <v/>
+      </c>
+      <c r="P60" s="40">
+        <f>IF(AND(ISNUMBER(Valuation!$C$35),Valuation!$C$35&gt;0),O60*(Valuation!$C$37/Valuation!$C$35),0)</f>
+        <v/>
+      </c>
+      <c r="Q60" s="22">
+        <f>IF(ISNUMBER(Valuation!$H$27),P60*Valuation!$H$27,0)</f>
+        <v/>
+      </c>
+      <c r="R60" s="70">
+        <f>IF(N60&gt;0,Q60/N60,0)</f>
+        <v/>
+      </c>
+      <c r="S60" s="40">
+        <f>IF(Q60&gt;0,IRR({-N60,0,0,0,0,Q60}),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Series A T1</t>
+        </is>
+      </c>
+      <c r="B61" s="39">
+        <f>'Cap Table'!C33</f>
+        <v/>
+      </c>
+      <c r="N61" s="10" t="n">
+        <v>500000</v>
+      </c>
+      <c r="O61" s="39">
+        <f>IF(Valuation!$C$34&gt;0,Valuation!$C$35*(N61/Valuation!$C$34),0)</f>
+        <v/>
+      </c>
+      <c r="P61" s="40">
+        <f>IF(AND(ISNUMBER(Valuation!$C$35),Valuation!$C$35&gt;0),O61*(Valuation!$C$37/Valuation!$C$35),0)</f>
+        <v/>
+      </c>
+      <c r="Q61" s="22">
+        <f>IF(ISNUMBER(Valuation!$H$27),P61*Valuation!$H$27,0)</f>
+        <v/>
+      </c>
+      <c r="R61" s="70">
+        <f>IF(N61&gt;0,Q61/N61,0)</f>
+        <v/>
+      </c>
+      <c r="S61" s="40">
+        <f>IF(Q61&gt;0,IRR({-N61,0,0,0,0,Q61}),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Series A T2</t>
+        </is>
+      </c>
+      <c r="B62" s="39">
+        <f>'Cap Table'!C34</f>
+        <v/>
+      </c>
+      <c r="N62" s="10" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="O62" s="39">
+        <f>IF(Valuation!$C$34&gt;0,Valuation!$C$35*(N62/Valuation!$C$34),0)</f>
+        <v/>
+      </c>
+      <c r="P62" s="40">
+        <f>IF(AND(ISNUMBER(Valuation!$C$35),Valuation!$C$35&gt;0),O62*(Valuation!$C$37/Valuation!$C$35),0)</f>
+        <v/>
+      </c>
+      <c r="Q62" s="22">
+        <f>IF(ISNUMBER(Valuation!$H$27),P62*Valuation!$H$27,0)</f>
+        <v/>
+      </c>
+      <c r="R62" s="70">
+        <f>IF(N62&gt;0,Q62/N62,0)</f>
+        <v/>
+      </c>
+      <c r="S62" s="40">
+        <f>IF(Q62&gt;0,IRR({-N62,0,0,0,0,Q62}),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Series B</t>
+        </is>
+      </c>
+      <c r="B63" s="39">
+        <f>'Cap Table'!C35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="71" t="inlineStr">
+        <is>
+          <t>Note: All charts update dynamically when the Scenario dropdown (Assumptions!C4) changes between Worst / Base / Best case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="18" t="inlineStr">
+        <is>
+          <t>Year (Extended)</t>
+        </is>
+      </c>
+      <c r="B80" s="18" t="inlineStr">
+        <is>
+          <t>Cum. Funds Raised</t>
+        </is>
+      </c>
+      <c r="C80" s="18" t="inlineStr">
+        <is>
+          <t>kWh Revenue (£)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="20" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B81" s="19">
+        <f>Scenarios!C12</f>
+        <v/>
+      </c>
+      <c r="C81" s="19">
+        <f>'Income Statement'!C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="20" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B82" s="19">
+        <f>Scenarios!D12</f>
+        <v/>
+      </c>
+      <c r="C82" s="19">
+        <f>'Income Statement'!D9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="20" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B83" s="19">
+        <f>Scenarios!E12</f>
+        <v/>
+      </c>
+      <c r="C83" s="19">
+        <f>'Income Statement'!E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="20" t="n">
+        <v>2029</v>
+      </c>
+      <c r="B84" s="19">
+        <f>Scenarios!F12</f>
+        <v/>
+      </c>
+      <c r="C84" s="19">
+        <f>'Income Statement'!F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="20" t="n">
+        <v>2030</v>
+      </c>
+      <c r="B85" s="19">
+        <f>Scenarios!G12</f>
+        <v/>
+      </c>
+      <c r="C85" s="19">
+        <f>'Income Statement'!G9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="n">
+        <v>2031</v>
+      </c>
+      <c r="B86" s="22">
+        <f>B85*(1+0.6)</f>
+        <v/>
+      </c>
+      <c r="C86" s="22">
+        <f>C85+B86*0.0212</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B87" s="22">
+        <f>B86*(1+0.6)</f>
+        <v/>
+      </c>
+      <c r="C87" s="22">
+        <f>C86+B87*0.0212</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="n">
+        <v>2033</v>
+      </c>
+      <c r="B88" s="22">
+        <f>B87*(1+0.6)</f>
+        <v/>
+      </c>
+      <c r="C88" s="22">
+        <f>C87+B88*0.0212</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B89" s="22">
+        <f>B88*(1+0.6)</f>
+        <v/>
+      </c>
+      <c r="C89" s="22">
+        <f>C88+B89*0.0212</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B90" s="22">
+        <f>B89*(1+0.6)</f>
+        <v/>
+      </c>
+      <c r="C90" s="22">
+        <f>C89+B90*0.0212</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="n">
+        <v>2036</v>
+      </c>
+      <c r="B91" s="22">
+        <f>B90*(1+0.6)</f>
+        <v/>
+      </c>
+      <c r="C91" s="22">
+        <f>C90+B91*0.0212</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="n">
+        <v>2037</v>
+      </c>
+      <c r="B92" s="22">
+        <f>B91*(1+0.6)</f>
+        <v/>
+      </c>
+      <c r="C92" s="22">
+        <f>C91+B92*0.0212</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="n">
+        <v>2038</v>
+      </c>
+      <c r="B93" s="22">
+        <f>B92*(1+0.6)</f>
+        <v/>
+      </c>
+      <c r="C93" s="22">
+        <f>C92+B93*0.0212</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="n">
+        <v>2039</v>
+      </c>
+      <c r="B94" s="22">
+        <f>B93*(1+0.6)</f>
+        <v/>
+      </c>
+      <c r="C94" s="22">
+        <f>C93+B94*0.0212</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="n">
+        <v>2040</v>
+      </c>
+      <c r="B95" s="22">
+        <f>B94*(1+0.6)</f>
+        <v/>
+      </c>
+      <c r="C95" s="22">
+        <f>C94+B95*0.0212</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="O42">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.3"/>
+        <cfvo type="num" val="0.5"/>
+        <color rgb="00FFC7CE"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00C6EFCE"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S58:S62">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.3"/>
+        <cfvo type="num" val="0.6"/>
+        <color rgb="00FFC7CE"/>
+        <color rgb="00FFEB9C"/>
+        <color rgb="00C6EFCE"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>